<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-24 15:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
@@ -182,7 +182,10 @@
     <t>cperez@zitron.com</t>
   </si>
   <si>
-    <t>MOTOR DE STOCK WEG - 02 POLOS - IE3 FRAME 280</t>
+    <t xml:space="preserve">Motores
+        OT 4324 — ZVN 1-7-37/2 – COD 350004
+        OT 4325 — ZVN 1-7-63/2 -- COD 350007
+</t>
   </si>
   <si>
     <t>Ingenieria Jefe de proyecto:,Analisis de costeo,propuesta motor OT 4324 4325</t>
@@ -191,34 +194,31 @@
     <t>Baja</t>
   </si>
   <si>
+    <t>1214969466296328</t>
+  </si>
+  <si>
+    <t>Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Selección de Rodete:
+        OT 4324 - Ventilador ZVN 1-7-37/2 --- COD. RODETE: 300059
+        OT 4325 - Ventilador ZVN 1-7-63/2 --- COD. RODETE: 300065
+</t>
+  </si>
+  <si>
+    <t>propuesta nucleo rodete OT 4324 4325,Ingenieria Jefe de proyecto:,Analisis de costeo,propuesta alabes OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969335257867</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:,Analisis de costeo,Planos preliminar</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1214969466296328</t>
-  </si>
-  <si>
-    <t>Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Selección de Rodete:
-        Rodete de placas s/plano 3073.00
-        Alabe s/ plano 3073.01
-        Z8 N600
-        Código 300003
-        hgutierrez@zitron.com, tu apoyo con la definición de calaje.
-</t>
-  </si>
-  <si>
-    <t>propuesta nucleo rodete OT 4324 4325,Ingenieria Jefe de proyecto:,Analisis de costeo,propuesta alabes OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969335257867</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:,Analisis de costeo,Planos preliminar</t>
   </si>
   <si>
     <t>1214969335257887</t>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46162.5836137963</v>
+        <v>46197.654548402774</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -2628,9 +2628,11 @@
       <c r="B11" s="9">
         <v>46162.55824909722</v>
       </c>
-      <c r="C11" s="10"/>
+      <c r="C11" s="9">
+        <v>46197.65242402778</v>
+      </c>
       <c r="D11" s="9">
-        <v>46196.60226733796</v>
+        <v>46197.65244247685</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>49</v>
@@ -2678,25 +2680,27 @@
         <v>54</v>
       </c>
       <c r="T11" s="10">
-        <v>0</v>
-      </c>
-      <c r="U11" s="12" t="s">
-        <v>55</v>
+        <v>1</v>
+      </c>
+      <c r="U11" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B12" s="5">
         <v>46162.55825447917</v>
       </c>
-      <c r="C12" s="6"/>
+      <c r="C12" s="5">
+        <v>46197.65454083333</v>
+      </c>
       <c r="D12" s="5">
-        <v>46175.874090578705</v>
+        <v>46197.654557013884</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>26</v>
@@ -2717,7 +2721,7 @@
         <v>26</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="M12" s="6" t="s">
         <v>26</v>
@@ -2729,7 +2733,7 @@
         <v>39</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q12" s="5">
         <v>46149</v>
@@ -2741,15 +2745,15 @@
         <v>54</v>
       </c>
       <c r="T12" s="6">
-        <v>0</v>
-      </c>
-      <c r="U12" s="12" t="s">
-        <v>55</v>
+        <v>1</v>
+      </c>
+      <c r="U12" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="9">
         <v>46162.55825988426</v>
@@ -2759,7 +2763,7 @@
         <v>46175.874089687495</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>26</v>
@@ -2792,7 +2796,7 @@
         <v>39</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q13" s="9">
         <v>46149</v>
@@ -2807,7 +2811,7 @@
         <v>0</v>
       </c>
       <c r="U13" s="12" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
@@ -2819,7 +2823,7 @@
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46162.664603599536</v>
+        <v>46197.65454884259</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>64</v>
@@ -2929,7 +2933,7 @@
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="5">
-        <v>46169.86243731482</v>
+        <v>46197.65244157407</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>71</v>
@@ -2979,8 +2983,8 @@
       <c r="T16" s="6">
         <v>0</v>
       </c>
-      <c r="U16" s="11" t="s">
-        <v>66</v>
+      <c r="U16" s="12" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
@@ -2992,7 +2996,7 @@
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="9">
-        <v>46169.862450347224</v>
+        <v>46197.654558842594</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>74</v>
@@ -3025,7 +3029,7 @@
         <v>68</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>75</v>
@@ -3042,8 +3046,8 @@
       <c r="T17" s="10">
         <v>0</v>
       </c>
-      <c r="U17" s="11" t="s">
-        <v>66</v>
+      <c r="U17" s="12" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
@@ -3057,7 +3061,7 @@
         <v>46197.58811052083</v>
       </c>
       <c r="D18" s="5">
-        <v>46197.588127407405</v>
+        <v>46197.654558912036</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>77</v>
@@ -3090,7 +3094,7 @@
         <v>68</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="P18" s="6" t="s">
         <v>79</v>
@@ -3107,8 +3111,8 @@
       <c r="T18" s="6">
         <v>1</v>
       </c>
-      <c r="U18" s="7" t="s">
-        <v>27</v>
+      <c r="U18" s="12" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
@@ -4842,7 +4846,7 @@
         <v>173</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P48" s="6" t="s">
         <v>179</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-25 16:39 UTC
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
@@ -2837,7 +2837,7 @@
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46197.58811732639</v>
+        <v>46198.68393108796</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>64</v>
@@ -2882,9 +2882,11 @@
       <c r="B15" s="9">
         <v>46162.55827298611</v>
       </c>
-      <c r="C15" s="10"/>
+      <c r="C15" s="9">
+        <v>46198.683924930556</v>
+      </c>
       <c r="D15" s="9">
-        <v>46197.65244157407</v>
+        <v>46198.683943310185</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>67</v>
@@ -2932,10 +2934,10 @@
         <v>54</v>
       </c>
       <c r="T15" s="10">
-        <v>0</v>
-      </c>
-      <c r="U15" s="12" t="s">
-        <v>47</v>
+        <v>1</v>
+      </c>
+      <c r="U15" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
@@ -3327,7 +3329,7 @@
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46162.59982563657</v>
+        <v>46198.68470386574</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>93</v>
@@ -3553,9 +3555,11 @@
       <c r="B26" s="5">
         <v>46162.558319710646</v>
       </c>
-      <c r="C26" s="6"/>
+      <c r="C26" s="5">
+        <v>46198.68469451389</v>
+      </c>
       <c r="D26" s="5">
-        <v>46169.86254357639</v>
+        <v>46198.684707002314</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>107</v>
@@ -3603,10 +3607,10 @@
         <v>54</v>
       </c>
       <c r="T26" s="6">
-        <v>0</v>
-      </c>
-      <c r="U26" s="11" t="s">
-        <v>82</v>
+        <v>1</v>
+      </c>
+      <c r="U26" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -3616,9 +3620,11 @@
       <c r="B27" s="9">
         <v>46162.55832415509</v>
       </c>
-      <c r="C27" s="10"/>
+      <c r="C27" s="9">
+        <v>46198.684641087966</v>
+      </c>
       <c r="D27" s="9">
-        <v>46197.58811881945</v>
+        <v>46198.68464270834</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>110</v>
@@ -3675,9 +3681,11 @@
       <c r="B28" s="5">
         <v>46162.5583337037</v>
       </c>
-      <c r="C28" s="6"/>
+      <c r="C28" s="5">
+        <v>46198.68467929398</v>
+      </c>
       <c r="D28" s="5">
-        <v>46169.86298305556</v>
+        <v>46198.68468228009</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>113</v>
@@ -3734,9 +3742,11 @@
       <c r="B29" s="9">
         <v>46162.55833876158</v>
       </c>
-      <c r="C29" s="10"/>
+      <c r="C29" s="9">
+        <v>46198.684322326386</v>
+      </c>
       <c r="D29" s="9">
-        <v>46196.17404179398</v>
+        <v>46198.684341354165</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>116</v>
@@ -3784,10 +3794,10 @@
         <v>33</v>
       </c>
       <c r="T29" s="10">
-        <v>0</v>
-      </c>
-      <c r="U29" s="11" t="s">
-        <v>82</v>
+        <v>1</v>
+      </c>
+      <c r="U29" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3797,9 +3807,11 @@
       <c r="B30" s="5">
         <v>46162.5583437037</v>
       </c>
-      <c r="C30" s="6"/>
+      <c r="C30" s="5">
+        <v>46198.68413635417</v>
+      </c>
       <c r="D30" s="5">
-        <v>46169.862896666666</v>
+        <v>46198.684137696764</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>119</v>
@@ -3856,9 +3868,11 @@
       <c r="B31" s="9">
         <v>46162.55834872685</v>
       </c>
-      <c r="C31" s="10"/>
+      <c r="C31" s="9">
+        <v>46198.68430692129</v>
+      </c>
       <c r="D31" s="9">
-        <v>46195.16988916667</v>
+        <v>46198.68430833334</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>122</v>
@@ -3915,9 +3929,11 @@
       <c r="B32" s="5">
         <v>46162.558353518514</v>
       </c>
-      <c r="C32" s="6"/>
+      <c r="C32" s="5">
+        <v>46198.68417550926</v>
+      </c>
       <c r="D32" s="5">
-        <v>46197.676590358795</v>
+        <v>46198.68417709491</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>125</v>
@@ -4829,7 +4845,7 @@
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46197.680058750004</v>
+        <v>46198.68419076389</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>178</v>
@@ -4879,8 +4895,8 @@
       <c r="T48" s="6">
         <v>0</v>
       </c>
-      <c r="U48" s="11" t="s">
-        <v>82</v>
+      <c r="U48" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
@@ -8244,7 +8260,7 @@
       </c>
       <c r="C111" s="10"/>
       <c r="D111" s="9">
-        <v>46162.673902361115</v>
+        <v>46198.68469991898</v>
       </c>
       <c r="E111" s="10" t="s">
         <v>298</v>
@@ -8294,8 +8310,8 @@
       <c r="T111" s="10">
         <v>0</v>
       </c>
-      <c r="U111" s="11" t="s">
-        <v>82</v>
+      <c r="U111" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
@@ -8370,7 +8386,7 @@
       </c>
       <c r="C113" s="10"/>
       <c r="D113" s="9">
-        <v>46197.17582074074</v>
+        <v>46198.684325486116</v>
       </c>
       <c r="E113" s="10" t="s">
         <v>304</v>
@@ -8420,8 +8436,8 @@
       <c r="T113" s="10">
         <v>0</v>
       </c>
-      <c r="U113" s="11" t="s">
-        <v>82</v>
+      <c r="U113" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-07-06 13:51 UTC
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2841" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2842" uniqueCount="513">
   <si>
     <t xml:space="preserve">50001553- ZITRON COLOMBIA ARIS MINING SEGOVIA - OT 4324 4325 </t>
   </si>
@@ -345,16 +345,16 @@
     <t>Fabricación Alabe OT 4324 4325,Generación OC Alabe OT 4324 4325</t>
   </si>
   <si>
+    <t>1214969379038319</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe OT 4324 4325,Alabe OT 4324 4325</t>
+  </si>
+  <si>
     <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1214969379038319</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe OT 4324 4325,Alabe OT 4324 4325</t>
   </si>
   <si>
     <t>1214969379038337</t>
@@ -2835,9 +2835,11 @@
       <c r="B14" s="5">
         <v>46162.55816920139</v>
       </c>
-      <c r="C14" s="6"/>
+      <c r="C14" s="5">
+        <v>46209.561731678245</v>
+      </c>
       <c r="D14" s="5">
-        <v>46206.5583869213</v>
+        <v>46209.56174483796</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>64</v>
@@ -2872,8 +2874,12 @@
       <c r="Q14" s="6"/>
       <c r="R14" s="6"/>
       <c r="S14" s="6"/>
-      <c r="T14" s="6"/>
-      <c r="U14" s="6"/>
+      <c r="T14" s="6">
+        <v>1</v>
+      </c>
+      <c r="U14" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
@@ -2947,9 +2953,11 @@
       <c r="B16" s="5">
         <v>46162.55827819444</v>
       </c>
-      <c r="C16" s="6"/>
+      <c r="C16" s="5">
+        <v>46209.56171221065</v>
+      </c>
       <c r="D16" s="5">
-        <v>46197.654558842594</v>
+        <v>46209.56277344907</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>70</v>
@@ -2997,10 +3005,10 @@
         <v>54</v>
       </c>
       <c r="T16" s="6">
-        <v>0</v>
-      </c>
-      <c r="U16" s="12" t="s">
-        <v>47</v>
+        <v>1</v>
+      </c>
+      <c r="U16" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
@@ -3014,7 +3022,7 @@
         <v>46197.58811052083</v>
       </c>
       <c r="D17" s="9">
-        <v>46197.77760189815</v>
+        <v>46209.5628121412</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>73</v>
@@ -3337,7 +3345,7 @@
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46198.68470386574</v>
+        <v>46209.56216927084</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>92</v>
@@ -3382,9 +3390,11 @@
       <c r="B23" s="9">
         <v>46162.558305694445</v>
       </c>
-      <c r="C23" s="10"/>
+      <c r="C23" s="9">
+        <v>46209.562155300926</v>
+      </c>
       <c r="D23" s="9">
-        <v>46169.86252686342</v>
+        <v>46209.563062939815</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>95</v>
@@ -3432,25 +3442,27 @@
         <v>54</v>
       </c>
       <c r="T23" s="10">
-        <v>0</v>
-      </c>
-      <c r="U23" s="11" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B24" s="5">
         <v>46162.55831018518</v>
       </c>
-      <c r="C24" s="6"/>
+      <c r="C24" s="5">
+        <v>46209.562107129634</v>
+      </c>
       <c r="D24" s="5">
-        <v>46169.86302510416</v>
+        <v>46209.56210862269</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
@@ -3483,7 +3495,7 @@
         <v>70</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
@@ -3494,7 +3506,7 @@
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -3504,9 +3516,11 @@
       <c r="B25" s="9">
         <v>46162.55831479166</v>
       </c>
-      <c r="C25" s="10"/>
+      <c r="C25" s="9">
+        <v>46209.562140995375</v>
+      </c>
       <c r="D25" s="9">
-        <v>46169.86304815972</v>
+        <v>46209.56214238426</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>104</v>
@@ -3539,7 +3553,7 @@
         <v>95</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P25" s="10" t="s">
         <v>105</v>
@@ -3553,7 +3567,7 @@
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
@@ -3567,7 +3581,7 @@
         <v>46198.68469451389</v>
       </c>
       <c r="D26" s="5">
-        <v>46198.684707002314</v>
+        <v>46209.563100486106</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>107</v>
@@ -3679,7 +3693,7 @@
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -3740,7 +3754,7 @@
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3866,7 +3880,7 @@
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -3927,7 +3941,7 @@
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -3988,7 +4002,7 @@
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
@@ -4051,7 +4065,7 @@
         <v>0</v>
       </c>
       <c r="U33" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -4110,7 +4124,7 @@
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -4169,7 +4183,7 @@
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -4232,7 +4246,7 @@
         <v>0</v>
       </c>
       <c r="U36" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -4401,7 +4415,7 @@
         <v>0</v>
       </c>
       <c r="U39" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
@@ -4623,7 +4637,7 @@
         <v>0</v>
       </c>
       <c r="U43" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -5034,7 +5048,7 @@
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -5756,7 +5770,7 @@
         <v>0</v>
       </c>
       <c r="U64" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -5819,7 +5833,7 @@
         <v>0</v>
       </c>
       <c r="U65" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
@@ -5882,7 +5896,7 @@
         <v>0</v>
       </c>
       <c r="U66" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -5945,7 +5959,7 @@
         <v>0</v>
       </c>
       <c r="U67" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -6008,7 +6022,7 @@
         <v>0</v>
       </c>
       <c r="U68" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -6071,7 +6085,7 @@
         <v>0</v>
       </c>
       <c r="U69" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
@@ -6181,7 +6195,7 @@
         <v>0</v>
       </c>
       <c r="U71" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -6880,7 +6894,7 @@
         <v>0</v>
       </c>
       <c r="U84" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
@@ -7579,7 +7593,7 @@
         <v>0</v>
       </c>
       <c r="U97" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
@@ -8337,7 +8351,7 @@
       </c>
       <c r="C112" s="6"/>
       <c r="D112" s="5">
-        <v>46162.673898912035</v>
+        <v>46209.562158773144</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>301</v>
@@ -8387,8 +8401,8 @@
       <c r="T112" s="6">
         <v>0</v>
       </c>
-      <c r="U112" s="11" t="s">
-        <v>99</v>
+      <c r="U112" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
@@ -8514,7 +8528,7 @@
         <v>0</v>
       </c>
       <c r="U114" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
@@ -8624,7 +8638,7 @@
         <v>0</v>
       </c>
       <c r="U116" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
@@ -9323,7 +9337,7 @@
         <v>0</v>
       </c>
       <c r="U129" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.25">
@@ -9998,7 +10012,7 @@
         <v>0</v>
       </c>
       <c r="U142" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
@@ -10697,7 +10711,7 @@
         <v>0</v>
       </c>
       <c r="U155" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="156" spans="1:21" x14ac:dyDescent="0.25">
@@ -11396,7 +11410,7 @@
         <v>0</v>
       </c>
       <c r="U168" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="169" spans="1:21" x14ac:dyDescent="0.25">
@@ -12071,7 +12085,7 @@
         <v>0</v>
       </c>
       <c r="U181" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="182" spans="1:21" x14ac:dyDescent="0.25">
@@ -12793,7 +12807,7 @@
         <v>0</v>
       </c>
       <c r="U195" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="196" spans="1:21" x14ac:dyDescent="0.25">
@@ -13468,7 +13482,7 @@
         <v>0</v>
       </c>
       <c r="U208" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="209" spans="1:21" x14ac:dyDescent="0.25">
@@ -14143,7 +14157,7 @@
         <v>0</v>
       </c>
       <c r="U221" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="222" spans="1:21" x14ac:dyDescent="0.25">
@@ -14818,7 +14832,7 @@
         <v>0</v>
       </c>
       <c r="U234" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="235" spans="1:21" x14ac:dyDescent="0.25">
@@ -15564,7 +15578,7 @@
         <v>0</v>
       </c>
       <c r="U248" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="249" spans="1:21" x14ac:dyDescent="0.25">
@@ -15627,7 +15641,7 @@
         <v>0</v>
       </c>
       <c r="U249" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-06 11:15 Chile
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
@@ -4362,9 +4362,11 @@
       <c r="B39" s="9">
         <v>46162.55843366898</v>
       </c>
-      <c r="C39" s="10"/>
+      <c r="C39" s="9">
+        <v>46209.612930856485</v>
+      </c>
       <c r="D39" s="9">
-        <v>46169.862598437496</v>
+        <v>46209.61294594908</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>147</v>
@@ -4412,10 +4414,10 @@
         <v>54</v>
       </c>
       <c r="T39" s="10">
-        <v>0</v>
-      </c>
-      <c r="U39" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U39" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
@@ -4425,9 +4427,11 @@
       <c r="B40" s="5">
         <v>46162.558437569445</v>
       </c>
-      <c r="C40" s="6"/>
+      <c r="C40" s="5">
+        <v>46209.6120780787</v>
+      </c>
       <c r="D40" s="5">
-        <v>46206.55996775463</v>
+        <v>46209.612079687504</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>90</v>
@@ -4478,9 +4482,11 @@
       <c r="B41" s="9">
         <v>46162.55844153935</v>
       </c>
-      <c r="C41" s="10"/>
+      <c r="C41" s="9">
+        <v>46209.61288494213</v>
+      </c>
       <c r="D41" s="9">
-        <v>46169.86272391204</v>
+        <v>46209.612886620365</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>154</v>
@@ -4533,7 +4539,7 @@
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46169.862742349535</v>
+        <v>46209.612896307866</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>157</v>
@@ -8477,7 +8483,7 @@
       </c>
       <c r="C114" s="6"/>
       <c r="D114" s="5">
-        <v>46162.67389181713</v>
+        <v>46209.61290208333</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>307</v>
@@ -8527,8 +8533,8 @@
       <c r="T114" s="6">
         <v>0</v>
       </c>
-      <c r="U114" s="11" t="s">
-        <v>102</v>
+      <c r="U114" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-07-06 21:31 UTC
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2842" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2843" uniqueCount="513">
   <si>
     <t xml:space="preserve">50001553- ZITRON COLOMBIA ARIS MINING SEGOVIA - OT 4324 4325 </t>
   </si>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46209.56216927084</v>
+        <v>46209.81432671296</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>92</v>
@@ -3381,7 +3381,9 @@
       <c r="R22" s="6"/>
       <c r="S22" s="6"/>
       <c r="T22" s="6"/>
-      <c r="U22" s="6"/>
+      <c r="U22" s="12" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
@@ -4012,9 +4014,11 @@
       <c r="B33" s="9">
         <v>46162.558358229166</v>
       </c>
-      <c r="C33" s="10"/>
+      <c r="C33" s="9">
+        <v>46209.81430680555</v>
+      </c>
       <c r="D33" s="9">
-        <v>46203.186885787036</v>
+        <v>46209.81431997685</v>
       </c>
       <c r="E33" s="10" t="s">
         <v>128</v>
@@ -4062,10 +4066,10 @@
         <v>33</v>
       </c>
       <c r="T33" s="10">
-        <v>0</v>
-      </c>
-      <c r="U33" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U33" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -4075,9 +4079,11 @@
       <c r="B34" s="5">
         <v>46162.5583628125</v>
       </c>
-      <c r="C34" s="6"/>
+      <c r="C34" s="5">
+        <v>46209.814144421296</v>
+      </c>
       <c r="D34" s="5">
-        <v>46206.55838853009</v>
+        <v>46209.814146226854</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>133</v>
@@ -4134,9 +4140,11 @@
       <c r="B35" s="9">
         <v>46162.55841275463</v>
       </c>
-      <c r="C35" s="10"/>
+      <c r="C35" s="9">
+        <v>46209.814290752314</v>
+      </c>
       <c r="D35" s="9">
-        <v>46202.16929391204</v>
+        <v>46209.8142920949</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>136</v>
@@ -4193,9 +4201,11 @@
       <c r="B36" s="5">
         <v>46162.558418622684</v>
       </c>
-      <c r="C36" s="6"/>
+      <c r="C36" s="5">
+        <v>46209.81447261574</v>
+      </c>
       <c r="D36" s="5">
-        <v>46203.186885821764</v>
+        <v>46209.81449996528</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>139</v>
@@ -4243,10 +4253,10 @@
         <v>33</v>
       </c>
       <c r="T36" s="6">
-        <v>0</v>
-      </c>
-      <c r="U36" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U36" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -4256,9 +4266,11 @@
       <c r="B37" s="9">
         <v>46162.558422118054</v>
       </c>
-      <c r="C37" s="10"/>
+      <c r="C37" s="9">
+        <v>46209.81440701389</v>
+      </c>
       <c r="D37" s="9">
-        <v>46206.559050254626</v>
+        <v>46209.81440909722</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>84</v>
@@ -4309,9 +4321,11 @@
       <c r="B38" s="5">
         <v>46162.558426400465</v>
       </c>
-      <c r="C38" s="6"/>
+      <c r="C38" s="5">
+        <v>46209.81445883102</v>
+      </c>
       <c r="D38" s="5">
-        <v>46171.17362893518</v>
+        <v>46209.81446026621</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>144</v>
@@ -4590,9 +4604,11 @@
       <c r="B43" s="9">
         <v>46162.55844833334</v>
       </c>
-      <c r="C43" s="10"/>
+      <c r="C43" s="9">
+        <v>46209.814689583334</v>
+      </c>
       <c r="D43" s="9">
-        <v>46203.186886435185</v>
+        <v>46209.81470094908</v>
       </c>
       <c r="E43" s="10" t="s">
         <v>161</v>
@@ -4640,10 +4656,10 @@
         <v>33</v>
       </c>
       <c r="T43" s="10">
-        <v>0</v>
-      </c>
-      <c r="U43" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U43" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -4653,9 +4669,11 @@
       <c r="B44" s="5">
         <v>46162.55845114583</v>
       </c>
-      <c r="C44" s="6"/>
+      <c r="C44" s="5">
+        <v>46209.814636689815</v>
+      </c>
       <c r="D44" s="5">
-        <v>46206.559488425926</v>
+        <v>46209.814638090276</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>87</v>
@@ -4706,9 +4724,11 @@
       <c r="B45" s="9">
         <v>46162.55845520833</v>
       </c>
-      <c r="C45" s="10"/>
+      <c r="C45" s="9">
+        <v>46209.81467625</v>
+      </c>
       <c r="D45" s="9">
-        <v>46202.16929168982</v>
+        <v>46209.81467782408</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>166</v>
@@ -5725,7 +5745,7 @@
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46204.167069814815</v>
+        <v>46209.81431027778</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>208</v>
@@ -5775,8 +5795,8 @@
       <c r="T64" s="6">
         <v>0</v>
       </c>
-      <c r="U64" s="11" t="s">
-        <v>102</v>
+      <c r="U64" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -5851,7 +5871,7 @@
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46204.16707040509</v>
+        <v>46209.814479583336</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>217</v>
@@ -5901,8 +5921,8 @@
       <c r="T66" s="6">
         <v>0</v>
       </c>
-      <c r="U66" s="11" t="s">
-        <v>102</v>
+      <c r="U66" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -5977,7 +5997,7 @@
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46204.1670715162</v>
+        <v>46209.814692500004</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>223</v>
@@ -6027,8 +6047,8 @@
       <c r="T68" s="6">
         <v>0</v>
       </c>
-      <c r="U68" s="11" t="s">
-        <v>102</v>
+      <c r="U68" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-08-13 20:59 UTC
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4324-4325.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2845" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2846" uniqueCount="511">
   <si>
     <t xml:space="preserve">50001553- ZITRON COLOMBIA ARIS MINING SEGOVIA - OT 4324 4325 </t>
   </si>
@@ -357,292 +357,292 @@
     <t>rodete OT 4324 4325,Materiales corte Laser OT 4324 4325,Alabe OT 4324 4325,Motor OT 4324 4325</t>
   </si>
   <si>
+    <t>1214969466331129</t>
+  </si>
+  <si>
+    <t>Alabe OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Eliana</t>
+  </si>
+  <si>
+    <t>ecarico@zitron.com</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe OT 4324 4325,Generación OC Alabe OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969379038319</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe OT 4324 4325,Alabe OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Tarea sin iniciar</t>
+  </si>
+  <si>
+    <t>1214969379038337</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Alabe OT 4324 4325,Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>1214969287532633</t>
+  </si>
+  <si>
+    <t>rodete OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete OT 4324 4325,Fabricación Rodete OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969287532648</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete OT 4324 4325</t>
+  </si>
+  <si>
+    <t>rodete OT 4324 4325,Fabricación Rodete OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969503994817</t>
+  </si>
+  <si>
+    <t>Fabricación Rodete OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Recepcion Rodete,rodete OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969504007335</t>
+  </si>
+  <si>
+    <t>Motor OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Generación OC motor OT 4324 4325,Fabricación motor OT 4324 4325,Planos motor proveedor OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969504007350</t>
+  </si>
+  <si>
+    <t>Generación OC motor OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Motor OT 4324 4325,Fabricación motor OT 4324 4325,Planos motor proveedor OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969504023948</t>
+  </si>
+  <si>
+    <t>Fabricación motor OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Recepcion motor,Motor OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969504023966</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Planos definitivos,Motor OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969335368176</t>
+  </si>
+  <si>
+    <t>Materiales corte Laser OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Yerlia Ayleen Castillo Diaz</t>
+  </si>
+  <si>
+    <t>yerlia.castillo@zitron.com</t>
+  </si>
+  <si>
+    <t>Fabricacion Corte Laser  OT 4324 4325,Generación OC materiales corte Laser OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969335368191</t>
+  </si>
+  <si>
+    <t>Generación OC materiales corte Laser OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Fabricacion Corte Laser  OT 4324 4325,Materiales corte Laser OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969379077262</t>
+  </si>
+  <si>
+    <t>Fabricacion Corte Laser  OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Recepcion materiales corte laser,Materiales corte Laser OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969379077280</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materiales Corte Plasma OT 4324 4325 </t>
+  </si>
+  <si>
+    <t>Generación OC Corte Plasma  OT 4324 4325,Fabricación Corte Plasma  OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969287605397</t>
+  </si>
+  <si>
+    <t>Materiales Corte Plasma OT 4324 4325 ,Fabricación Corte Plasma  OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969287605412</t>
+  </si>
+  <si>
+    <t>Fabricación Corte Plasma  OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Materiales Corte Plasma OT 4324 4325 ,Recepcion Materiales corte plasma</t>
+  </si>
+  <si>
+    <t>1214969287605814</t>
+  </si>
+  <si>
+    <t>Fabricación Externa  OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Rosemary Singh</t>
+  </si>
+  <si>
+    <t>rosemary.singh@zitron.com</t>
+  </si>
+  <si>
+    <t>Generacion OC Fabricación Externa OT 4324 4325,Fabricación estructura proveedor externo OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969287605824</t>
+  </si>
+  <si>
+    <t>Fabricación Externa  OT 4324 4325,Fabricación estructura proveedor externo OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969287605839</t>
+  </si>
+  <si>
+    <t>Fabricación estructura proveedor externo OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Recepcion fabricación externa ,Fabricación Externa  OT 4324 4325,Control de calidad fabricación externa  OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969466515947</t>
+  </si>
+  <si>
+    <t>Control de calidad fabricación externa  OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Nicolás López</t>
+  </si>
+  <si>
+    <t>nicolas.lopez@zitron.com</t>
+  </si>
+  <si>
+    <t>1214969466515957</t>
+  </si>
+  <si>
+    <t>Mecanizado OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Generación OC Mecanizado OT 4324 4325,Fabricación Mecanizado OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969466515967</t>
+  </si>
+  <si>
+    <t>Mecanizado OT 4324 4325,Fabricación Mecanizado OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969335445666</t>
+  </si>
+  <si>
+    <t>Fabricación Mecanizado OT 4324 4325</t>
+  </si>
+  <si>
+    <t>Recepcion mecanizado,Mecanizado OT 4324 4325</t>
+  </si>
+  <si>
+    <t>1214969284200803</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseñoo:</t>
+  </si>
+  <si>
+    <t>Planos preliminar,Planos definitivos</t>
+  </si>
+  <si>
+    <t>1214969335445681</t>
+  </si>
+  <si>
+    <t>Planos preliminar</t>
+  </si>
+  <si>
+    <t>Gonzalo Javier Dávila Bade</t>
+  </si>
+  <si>
+    <t>gonzalo.davila@zitron.com</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseñoo:,Planos definitivos</t>
+  </si>
+  <si>
+    <t>1214969466529004</t>
+  </si>
+  <si>
+    <t>Planos definitivos</t>
+  </si>
+  <si>
+    <t>Planos preliminar,Planos motor proveedor OT 4324 4325</t>
+  </si>
+  <si>
+    <t>check planos,Ingenieria y diseñoo:</t>
+  </si>
+  <si>
+    <t>1214969379162030</t>
+  </si>
+  <si>
+    <t>Hernan Roberto Gutierrez Barrientos</t>
+  </si>
+  <si>
+    <t>hgutierrez@zitron.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4325- ZVN 1-7-63/2,OT 4325- ZVN 1-7-63/2,OT 4325- ZVN 1-7-63/2,OT 4325- ZVN 1-7-63/2,OT 4325- ZVN 1-7-63/2,OT 4324- ZVN 1-7-37/2 ,Propuesta Mecanizado OT 4324 4325,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,Propuesta Fabricación externa  OT 4324 4325,propuesta Corte Laser OT 4324 4325,Propuesta Corte plasma  OT 4324 4325,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 </t>
+  </si>
+  <si>
+    <t>1214969335458365</t>
+  </si>
+  <si>
+    <t>check pruebas FAT</t>
+  </si>
+  <si>
+    <t>Francisca González Cornejo</t>
+  </si>
+  <si>
+    <t>francisca.gonzalez@zitron.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 </t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1214969466331129</t>
-  </si>
-  <si>
-    <t>Alabe OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Eliana</t>
-  </si>
-  <si>
-    <t>ecarico@zitron.com</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe OT 4324 4325,Generación OC Alabe OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969379038319</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe OT 4324 4325,Alabe OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1214969379038337</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Alabe OT 4324 4325,Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>1214969287532633</t>
-  </si>
-  <si>
-    <t>rodete OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete OT 4324 4325,Fabricación Rodete OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969287532648</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete OT 4324 4325</t>
-  </si>
-  <si>
-    <t>rodete OT 4324 4325,Fabricación Rodete OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969503994817</t>
-  </si>
-  <si>
-    <t>Fabricación Rodete OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Recepcion Rodete,rodete OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969504007335</t>
-  </si>
-  <si>
-    <t>Motor OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Generación OC motor OT 4324 4325,Fabricación motor OT 4324 4325,Planos motor proveedor OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969504007350</t>
-  </si>
-  <si>
-    <t>Generación OC motor OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Motor OT 4324 4325,Fabricación motor OT 4324 4325,Planos motor proveedor OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969504023948</t>
-  </si>
-  <si>
-    <t>Fabricación motor OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Recepcion motor,Motor OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969504023966</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Planos definitivos,Motor OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969335368176</t>
-  </si>
-  <si>
-    <t>Materiales corte Laser OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Yerlia Ayleen Castillo Diaz</t>
-  </si>
-  <si>
-    <t>yerlia.castillo@zitron.com</t>
-  </si>
-  <si>
-    <t>Fabricacion Corte Laser  OT 4324 4325,Generación OC materiales corte Laser OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969335368191</t>
-  </si>
-  <si>
-    <t>Generación OC materiales corte Laser OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Fabricacion Corte Laser  OT 4324 4325,Materiales corte Laser OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969379077262</t>
-  </si>
-  <si>
-    <t>Fabricacion Corte Laser  OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Recepcion materiales corte laser,Materiales corte Laser OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969379077280</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Materiales Corte Plasma OT 4324 4325 </t>
-  </si>
-  <si>
-    <t>Generación OC Corte Plasma  OT 4324 4325,Fabricación Corte Plasma  OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969287605397</t>
-  </si>
-  <si>
-    <t>Materiales Corte Plasma OT 4324 4325 ,Fabricación Corte Plasma  OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969287605412</t>
-  </si>
-  <si>
-    <t>Fabricación Corte Plasma  OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Materiales Corte Plasma OT 4324 4325 ,Recepcion Materiales corte plasma</t>
-  </si>
-  <si>
-    <t>1214969287605814</t>
-  </si>
-  <si>
-    <t>Fabricación Externa  OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Rosemary Singh</t>
-  </si>
-  <si>
-    <t>rosemary.singh@zitron.com</t>
-  </si>
-  <si>
-    <t>Generacion OC Fabricación Externa OT 4324 4325,Fabricación estructura proveedor externo OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969287605824</t>
-  </si>
-  <si>
-    <t>Fabricación Externa  OT 4324 4325,Fabricación estructura proveedor externo OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969287605839</t>
-  </si>
-  <si>
-    <t>Fabricación estructura proveedor externo OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Recepcion fabricación externa ,Fabricación Externa  OT 4324 4325,Control de calidad fabricación externa  OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969466515947</t>
-  </si>
-  <si>
-    <t>Control de calidad fabricación externa  OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Nicolás López</t>
-  </si>
-  <si>
-    <t>nicolas.lopez@zitron.com</t>
-  </si>
-  <si>
-    <t>1214969466515957</t>
-  </si>
-  <si>
-    <t>Mecanizado OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Generación OC Mecanizado OT 4324 4325,Fabricación Mecanizado OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969466515967</t>
-  </si>
-  <si>
-    <t>Mecanizado OT 4324 4325,Fabricación Mecanizado OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969335445666</t>
-  </si>
-  <si>
-    <t>Fabricación Mecanizado OT 4324 4325</t>
-  </si>
-  <si>
-    <t>Recepcion mecanizado,Mecanizado OT 4324 4325</t>
-  </si>
-  <si>
-    <t>1214969284200803</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseñoo:</t>
-  </si>
-  <si>
-    <t>Planos preliminar,Planos definitivos</t>
-  </si>
-  <si>
-    <t>1214969335445681</t>
-  </si>
-  <si>
-    <t>Planos preliminar</t>
-  </si>
-  <si>
-    <t>Gonzalo Javier Dávila Bade</t>
-  </si>
-  <si>
-    <t>gonzalo.davila@zitron.com</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseñoo:,Planos definitivos</t>
-  </si>
-  <si>
-    <t>1214969466529004</t>
-  </si>
-  <si>
-    <t>Planos definitivos</t>
-  </si>
-  <si>
-    <t>Planos preliminar,Planos motor proveedor OT 4324 4325</t>
-  </si>
-  <si>
-    <t>check planos,Ingenieria y diseñoo:</t>
-  </si>
-  <si>
-    <t>1214969379162030</t>
-  </si>
-  <si>
-    <t>Hernan Roberto Gutierrez Barrientos</t>
-  </si>
-  <si>
-    <t>hgutierrez@zitron.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4325- ZVN 1-7-63/2,OT 4325- ZVN 1-7-63/2,OT 4325- ZVN 1-7-63/2,OT 4325- ZVN 1-7-63/2,OT 4325- ZVN 1-7-63/2,OT 4324- ZVN 1-7-37/2 ,Propuesta Mecanizado OT 4324 4325,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,Propuesta Fabricación externa  OT 4324 4325,propuesta Corte Laser OT 4324 4325,Propuesta Corte plasma  OT 4324 4325,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 </t>
-  </si>
-  <si>
-    <t>1214969335458365</t>
-  </si>
-  <si>
-    <t>check pruebas FAT</t>
-  </si>
-  <si>
-    <t>Francisca González Cornejo</t>
-  </si>
-  <si>
-    <t>francisca.gonzalez@zitron.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4324- ZVN 1-7-37/2 ,OT 4324- ZVN 1-7-37/2 </t>
   </si>
   <si>
     <t>1214969335458375</t>
@@ -3371,9 +3371,11 @@
       <c r="B22" s="5">
         <v>46162.55817344907</v>
       </c>
-      <c r="C22" s="6"/>
+      <c r="C22" s="5">
+        <v>46247.81442592593</v>
+      </c>
       <c r="D22" s="5">
-        <v>46209.81432671296</v>
+        <v>46247.81443989583</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>91</v>
@@ -3408,14 +3410,16 @@
       <c r="Q22" s="6"/>
       <c r="R22" s="6"/>
       <c r="S22" s="6"/>
-      <c r="T22" s="6"/>
-      <c r="U22" s="12" t="s">
-        <v>93</v>
+      <c r="T22" s="6">
+        <v>1</v>
+      </c>
+      <c r="U22" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B23" s="9">
         <v>46162.558305694445</v>
@@ -3427,16 +3431,16 @@
         <v>46209.563062939815</v>
       </c>
       <c r="E23" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="F23" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G23" s="10" t="s">
+      <c r="H23" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>97</v>
       </c>
       <c r="I23" s="9">
         <v>46155</v>
@@ -3457,7 +3461,7 @@
         <v>91</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P23" s="10" t="s">
         <v>91</v>
@@ -3480,7 +3484,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B24" s="5">
         <v>46162.55831018518</v>
@@ -3492,16 +3496,16 @@
         <v>46209.56210862269</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>97</v>
       </c>
       <c r="I24" s="5">
         <v>46155</v>
@@ -3519,13 +3523,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O24" s="6" t="s">
         <v>70</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
@@ -3536,12 +3540,12 @@
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B25" s="9">
         <v>46162.55831479166</v>
@@ -3553,16 +3557,16 @@
         <v>46209.56214238426</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>97</v>
       </c>
       <c r="I25" s="9">
         <v>46157</v>
@@ -3580,13 +3584,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
@@ -3597,12 +3601,12 @@
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B26" s="5">
         <v>46162.558319710646</v>
@@ -3614,16 +3618,16 @@
         <v>46209.563100486106</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>97</v>
       </c>
       <c r="I26" s="5">
         <v>46155</v>
@@ -3644,7 +3648,7 @@
         <v>91</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>91</v>
@@ -3667,7 +3671,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B27" s="9">
         <v>46162.55832415509</v>
@@ -3679,16 +3683,16 @@
         <v>46198.68464270834</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="H27" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>97</v>
       </c>
       <c r="I27" s="9">
         <v>46155</v>
@@ -3706,13 +3710,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O27" s="10" t="s">
         <v>73</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
@@ -3723,12 +3727,12 @@
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B28" s="5">
         <v>46162.5583337037</v>
@@ -3740,16 +3744,16 @@
         <v>46198.68468228009</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>97</v>
       </c>
       <c r="I28" s="5">
         <v>46157</v>
@@ -3767,13 +3771,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
@@ -3784,12 +3788,12 @@
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B29" s="9">
         <v>46162.55833876158</v>
@@ -3801,16 +3805,16 @@
         <v>46198.684341354165</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="H29" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="H29" s="10" t="s">
-        <v>97</v>
       </c>
       <c r="I29" s="9">
         <v>46155</v>
@@ -3831,7 +3835,7 @@
         <v>91</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="P29" s="10" t="s">
         <v>91</v>
@@ -3854,7 +3858,7 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B30" s="5">
         <v>46162.5583437037</v>
@@ -3866,16 +3870,16 @@
         <v>46198.684137696764</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>97</v>
       </c>
       <c r="I30" s="5">
         <v>46155</v>
@@ -3893,13 +3897,13 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>67</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
@@ -3910,12 +3914,12 @@
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B31" s="9">
         <v>46162.55834872685</v>
@@ -3927,16 +3931,16 @@
         <v>46198.68430833334</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="H31" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="H31" s="10" t="s">
-        <v>97</v>
       </c>
       <c r="I31" s="9">
         <v>46167</v>
@@ -3954,13 +3958,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
@@ -3971,12 +3975,12 @@
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B32" s="5">
         <v>46162.558353518514</v>
@@ -3988,16 +3992,16 @@
         <v>46198.68417709491</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>97</v>
       </c>
       <c r="I32" s="5">
         <v>46167</v>
@@ -4015,13 +4019,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
@@ -4032,12 +4036,12 @@
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B33" s="9">
         <v>46162.558358229166</v>
@@ -4049,16 +4053,16 @@
         <v>46209.81431997685</v>
       </c>
       <c r="E33" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G33" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F33" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G33" s="10" t="s">
+      <c r="H33" s="10" t="s">
         <v>129</v>
-      </c>
-      <c r="H33" s="10" t="s">
-        <v>130</v>
       </c>
       <c r="I33" s="9">
         <v>46190</v>
@@ -4079,7 +4083,7 @@
         <v>91</v>
       </c>
       <c r="O33" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P33" s="10" t="s">
         <v>91</v>
@@ -4102,7 +4106,7 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B34" s="5">
         <v>46162.5583628125</v>
@@ -4114,16 +4118,16 @@
         <v>46209.814146226854</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>130</v>
       </c>
       <c r="I34" s="5">
         <v>46190</v>
@@ -4141,13 +4145,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>78</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
@@ -4158,12 +4162,12 @@
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B35" s="9">
         <v>46162.55841275463</v>
@@ -4175,16 +4179,16 @@
         <v>46209.8142920949</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="H35" s="10" t="s">
         <v>129</v>
-      </c>
-      <c r="H35" s="10" t="s">
-        <v>130</v>
       </c>
       <c r="I35" s="9">
         <v>46192</v>
@@ -4202,13 +4206,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
@@ -4219,12 +4223,12 @@
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B36" s="5">
         <v>46162.558418622684</v>
@@ -4236,16 +4240,16 @@
         <v>46209.81449996528</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>130</v>
       </c>
       <c r="I36" s="5">
         <v>46190</v>
@@ -4266,7 +4270,7 @@
         <v>91</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>26</v>
@@ -4289,7 +4293,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B37" s="9">
         <v>46162.558422118054</v>
@@ -4307,10 +4311,10 @@
         <v>26</v>
       </c>
       <c r="G37" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="H37" s="10" t="s">
         <v>129</v>
-      </c>
-      <c r="H37" s="10" t="s">
-        <v>130</v>
       </c>
       <c r="I37" s="9">
         <v>46190</v>
@@ -4328,13 +4332,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="O37" s="10" t="s">
         <v>82</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
@@ -4344,7 +4348,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B38" s="5">
         <v>46162.558426400465</v>
@@ -4356,16 +4360,16 @@
         <v>46209.81446026621</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="H38" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>130</v>
       </c>
       <c r="I38" s="5">
         <v>46161</v>
@@ -4383,13 +4387,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="O38" s="6" t="s">
         <v>83</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -4399,7 +4403,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B39" s="9">
         <v>46162.55843366898</v>
@@ -4411,16 +4415,16 @@
         <v>46232.17963666667</v>
       </c>
       <c r="E39" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G39" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="F39" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G39" s="10" t="s">
+      <c r="H39" s="10" t="s">
         <v>148</v>
-      </c>
-      <c r="H39" s="10" t="s">
-        <v>149</v>
       </c>
       <c r="I39" s="9">
         <v>46190</v>
@@ -4441,7 +4445,7 @@
         <v>91</v>
       </c>
       <c r="O39" s="10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P39" s="10" t="s">
         <v>26</v>
@@ -4464,7 +4468,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B40" s="5">
         <v>46162.558437569445</v>
@@ -4482,10 +4486,10 @@
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>148</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>149</v>
       </c>
       <c r="I40" s="5">
         <v>46190</v>
@@ -4503,13 +4507,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>88</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
@@ -4519,7 +4523,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B41" s="9">
         <v>46162.55844153935</v>
@@ -4531,16 +4535,16 @@
         <v>46209.612886620365</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="H41" s="10" t="s">
         <v>148</v>
-      </c>
-      <c r="H41" s="10" t="s">
-        <v>149</v>
       </c>
       <c r="I41" s="9">
         <v>46199</v>
@@ -4558,13 +4562,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="O41" s="10" t="s">
         <v>89</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="Q41" s="10"/>
       <c r="R41" s="10"/>
@@ -4574,7 +4578,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B42" s="5">
         <v>46162.55844576389</v>
@@ -4586,16 +4590,16 @@
         <v>46216.54443384259</v>
       </c>
       <c r="E42" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G42" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="F42" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G42" s="6" t="s">
+      <c r="H42" s="6" t="s">
         <v>158</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>159</v>
       </c>
       <c r="I42" s="5">
         <v>46230</v>
@@ -4613,10 +4617,10 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>26</v>
@@ -4629,7 +4633,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B43" s="9">
         <v>46162.55844833334</v>
@@ -4641,16 +4645,16 @@
         <v>46209.81470094908</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="H43" s="10" t="s">
         <v>129</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>130</v>
       </c>
       <c r="I43" s="9">
         <v>46190</v>
@@ -4671,7 +4675,7 @@
         <v>91</v>
       </c>
       <c r="O43" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="P43" s="10" t="s">
         <v>26</v>
@@ -4694,7 +4698,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B44" s="5">
         <v>46162.55845114583</v>
@@ -4712,10 +4716,10 @@
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="H44" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>130</v>
       </c>
       <c r="I44" s="5">
         <v>46190</v>
@@ -4733,13 +4737,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>85</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4749,7 +4753,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B45" s="9">
         <v>46162.55845520833</v>
@@ -4761,16 +4765,16 @@
         <v>46209.81467782408</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="H45" s="10" t="s">
         <v>129</v>
-      </c>
-      <c r="H45" s="10" t="s">
-        <v>130</v>
       </c>
       <c r="I45" s="9">
         <v>46192</v>
@@ -4788,13 +4792,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O45" s="10" t="s">
         <v>86</v>
       </c>
       <c r="P45" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="Q45" s="10"/>
       <c r="R45" s="10"/>
@@ -4804,7 +4808,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B46" s="5">
         <v>46162.55817767361</v>
@@ -4816,7 +4820,7 @@
         <v>46210.528923819445</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>25</v>
@@ -4840,7 +4844,7 @@
         <v>26</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>26</v>
@@ -4857,7 +4861,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B47" s="9">
         <v>46162.55845957176</v>
@@ -4869,16 +4873,16 @@
         <v>46197.67690475694</v>
       </c>
       <c r="E47" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G47" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="F47" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G47" s="10" t="s">
+      <c r="H47" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="H47" s="10" t="s">
-        <v>174</v>
       </c>
       <c r="I47" s="9">
         <v>46160</v>
@@ -4896,13 +4900,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O47" s="10" t="s">
         <v>60</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="Q47" s="9">
         <v>46160</v>
@@ -4922,7 +4926,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B48" s="5">
         <v>46162.55846439815</v>
@@ -4934,16 +4938,16 @@
         <v>46198.79333422454</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="H48" s="6" t="s">
         <v>173</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>174</v>
       </c>
       <c r="I48" s="5">
         <v>46176</v>
@@ -4961,13 +4965,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O48" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="P48" s="6" t="s">
         <v>178</v>
-      </c>
-      <c r="P48" s="6" t="s">
-        <v>179</v>
       </c>
       <c r="Q48" s="5">
         <v>46176</v>
@@ -4987,7 +4991,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B49" s="9">
         <v>46162.55847024306</v>
@@ -5005,10 +5009,10 @@
         <v>26</v>
       </c>
       <c r="G49" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="H49" s="10" t="s">
         <v>181</v>
-      </c>
-      <c r="H49" s="10" t="s">
-        <v>182</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="9">
@@ -5024,13 +5028,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O49" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="P49" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Q49" s="9">
         <v>46185</v>
@@ -5050,26 +5054,28 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B50" s="5">
         <v>46162.55848571759</v>
       </c>
-      <c r="C50" s="6"/>
+      <c r="C50" s="5">
+        <v>46247.81199479167</v>
+      </c>
       <c r="D50" s="5">
-        <v>46226.20215001157</v>
+        <v>46247.813050763885</v>
       </c>
       <c r="E50" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G50" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F50" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G50" s="6" t="s">
+      <c r="H50" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="I50" s="5">
         <v>46225</v>
@@ -5087,10 +5093,10 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>26</v>
@@ -5105,10 +5111,10 @@
         <v>33</v>
       </c>
       <c r="T50" s="6">
-        <v>0</v>
-      </c>
-      <c r="U50" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U50" s="12" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -5118,9 +5124,11 @@
       <c r="B51" s="9">
         <v>46162.5584890162</v>
       </c>
-      <c r="C51" s="10"/>
+      <c r="C51" s="9">
+        <v>46247.81167303241</v>
+      </c>
       <c r="D51" s="9">
-        <v>46225.16841835648</v>
+        <v>46247.814428935184</v>
       </c>
       <c r="E51" s="10" t="s">
         <v>190</v>
@@ -5129,10 +5137,10 @@
         <v>26</v>
       </c>
       <c r="G51" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="H51" s="10" t="s">
         <v>186</v>
-      </c>
-      <c r="H51" s="10" t="s">
-        <v>187</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="9">
@@ -5148,7 +5156,7 @@
         <v>26</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O51" s="10" t="s">
         <v>190</v>
@@ -5169,9 +5177,11 @@
       <c r="B52" s="5">
         <v>46162.558492951386</v>
       </c>
-      <c r="C52" s="6"/>
+      <c r="C52" s="5">
+        <v>46247.81303396991</v>
+      </c>
       <c r="D52" s="5">
-        <v>46225.16841996528</v>
+        <v>46247.81442918981</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>190</v>
@@ -5180,10 +5190,10 @@
         <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="H52" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="I52" s="6"/>
       <c r="J52" s="5">
@@ -5199,7 +5209,7 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>190</v>
@@ -5220,9 +5230,11 @@
       <c r="B53" s="9">
         <v>46162.55849660879</v>
       </c>
-      <c r="C53" s="10"/>
+      <c r="C53" s="9">
+        <v>46247.814462696755</v>
+      </c>
       <c r="D53" s="9">
-        <v>46225.168421215276</v>
+        <v>46247.81446421296</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>190</v>
@@ -5231,10 +5243,10 @@
         <v>26</v>
       </c>
       <c r="G53" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="H53" s="10" t="s">
         <v>186</v>
-      </c>
-      <c r="H53" s="10" t="s">
-        <v>187</v>
       </c>
       <c r="I53" s="10"/>
       <c r="J53" s="9">
@@ -5250,7 +5262,7 @@
         <v>26</v>
       </c>
       <c r="N53" s="10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O53" s="10" t="s">
         <v>190</v>
@@ -5271,9 +5283,11 @@
       <c r="B54" s="5">
         <v>46162.55849916667</v>
       </c>
-      <c r="C54" s="6"/>
+      <c r="C54" s="5">
+        <v>46247.81451542824</v>
+      </c>
       <c r="D54" s="5">
-        <v>46225.16838393519</v>
+        <v>46247.81452064815</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>190</v>
@@ -5282,10 +5296,10 @@
         <v>26</v>
       </c>
       <c r="G54" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="H54" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="H54" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="I54" s="6"/>
       <c r="J54" s="5">
@@ -5301,7 +5315,7 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>190</v>
@@ -5322,9 +5336,11 @@
       <c r="B55" s="9">
         <v>46162.55850175926</v>
       </c>
-      <c r="C55" s="10"/>
+      <c r="C55" s="9">
+        <v>46247.81451621528</v>
+      </c>
       <c r="D55" s="9">
-        <v>46225.16838541666</v>
+        <v>46247.81452103009</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>196</v>
@@ -5333,10 +5349,10 @@
         <v>26</v>
       </c>
       <c r="G55" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="H55" s="10" t="s">
         <v>186</v>
-      </c>
-      <c r="H55" s="10" t="s">
-        <v>187</v>
       </c>
       <c r="I55" s="10"/>
       <c r="J55" s="9">
@@ -5352,7 +5368,7 @@
         <v>26</v>
       </c>
       <c r="N55" s="10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O55" s="10" t="s">
         <v>196</v>
@@ -5373,9 +5389,11 @@
       <c r="B56" s="5">
         <v>46162.56211614583</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46247.81451681713</v>
+      </c>
       <c r="D56" s="5">
-        <v>46225.16840149305</v>
+        <v>46247.81452143518</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>196</v>
@@ -5384,10 +5402,10 @@
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="H56" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="I56" s="6"/>
       <c r="J56" s="5">
@@ -5403,7 +5421,7 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>196</v>
@@ -5424,9 +5442,11 @@
       <c r="B57" s="9">
         <v>46162.56212396991</v>
       </c>
-      <c r="C57" s="10"/>
+      <c r="C57" s="9">
+        <v>46247.814517210645</v>
+      </c>
       <c r="D57" s="9">
-        <v>46225.16840322917</v>
+        <v>46247.81452175926</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>196</v>
@@ -5435,10 +5455,10 @@
         <v>26</v>
       </c>
       <c r="G57" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="H57" s="10" t="s">
         <v>186</v>
-      </c>
-      <c r="H57" s="10" t="s">
-        <v>187</v>
       </c>
       <c r="I57" s="10"/>
       <c r="J57" s="9">
@@ -5454,7 +5474,7 @@
         <v>26</v>
       </c>
       <c r="N57" s="10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O57" s="10" t="s">
         <v>196</v>
@@ -5475,9 +5495,11 @@
       <c r="B58" s="5">
         <v>46162.56213497685</v>
       </c>
-      <c r="C58" s="6"/>
+      <c r="C58" s="5">
+        <v>46247.814517743056</v>
+      </c>
       <c r="D58" s="5">
-        <v>46225.16840447916</v>
+        <v>46247.81452204861</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>196</v>
@@ -5486,10 +5508,10 @@
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="H58" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="H58" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="I58" s="6"/>
       <c r="J58" s="5">
@@ -5505,7 +5527,7 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>196</v>
@@ -5526,9 +5548,11 @@
       <c r="B59" s="9">
         <v>46162.562155057865</v>
       </c>
-      <c r="C59" s="10"/>
+      <c r="C59" s="9">
+        <v>46247.814518263884</v>
+      </c>
       <c r="D59" s="9">
-        <v>46225.16840631944</v>
+        <v>46247.81452231482</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>196</v>
@@ -5537,10 +5561,10 @@
         <v>26</v>
       </c>
       <c r="G59" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="H59" s="10" t="s">
         <v>186</v>
-      </c>
-      <c r="H59" s="10" t="s">
-        <v>187</v>
       </c>
       <c r="I59" s="10"/>
       <c r="J59" s="9">
@@ -5556,7 +5580,7 @@
         <v>26</v>
       </c>
       <c r="N59" s="10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O59" s="10" t="s">
         <v>196</v>
@@ -5577,9 +5601,11 @@
       <c r="B60" s="5">
         <v>46162.562163055554</v>
       </c>
-      <c r="C60" s="6"/>
+      <c r="C60" s="5">
+        <v>46247.81451863426</v>
+      </c>
       <c r="D60" s="5">
-        <v>46225.1684090625</v>
+        <v>46247.81452263889</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>196</v>
@@ -5588,10 +5614,10 @@
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="H60" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="H60" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="I60" s="6"/>
       <c r="J60" s="5">
@@ -5607,7 +5633,7 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>196</v>
@@ -5628,9 +5654,11 @@
       <c r="B61" s="9">
         <v>46162.56217104167</v>
       </c>
-      <c r="C61" s="10"/>
+      <c r="C61" s="9">
+        <v>46247.81451899305</v>
+      </c>
       <c r="D61" s="9">
-        <v>46225.168411701394</v>
+        <v>46247.81452295139</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>196</v>
@@ -5639,10 +5667,10 @@
         <v>26</v>
       </c>
       <c r="G61" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="H61" s="10" t="s">
         <v>186</v>
-      </c>
-      <c r="H61" s="10" t="s">
-        <v>187</v>
       </c>
       <c r="I61" s="10"/>
       <c r="J61" s="9">
@@ -5658,7 +5686,7 @@
         <v>26</v>
       </c>
       <c r="N61" s="10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O61" s="10" t="s">
         <v>196</v>
@@ -5679,9 +5707,11 @@
       <c r="B62" s="5">
         <v>46162.562178935186</v>
       </c>
-      <c r="C62" s="6"/>
+      <c r="C62" s="5">
+        <v>46247.81451936343</v>
+      </c>
       <c r="D62" s="5">
-        <v>46225.16841293982</v>
+        <v>46247.81452326389</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>196</v>
@@ -5690,10 +5720,10 @@
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="H62" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="H62" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="I62" s="6"/>
       <c r="J62" s="5">
@@ -5709,7 +5739,7 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>196</v>
@@ -5820,7 +5850,7 @@
         <v>205</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P64" s="6" t="s">
         <v>211</v>
@@ -5861,10 +5891,10 @@
         <v>26</v>
       </c>
       <c r="G65" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H65" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="H65" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="I65" s="9">
         <v>46204</v>
@@ -5950,7 +5980,7 @@
         <v>205</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>218</v>
@@ -5991,10 +6021,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H67" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="H67" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="I67" s="9">
         <v>46204</v>
@@ -6080,7 +6110,7 @@
         <v>205</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P68" s="6" t="s">
         <v>223</v>
@@ -6121,10 +6151,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H69" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="H69" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="I69" s="9">
         <v>46204</v>
@@ -6173,9 +6203,11 @@
       <c r="B70" s="5">
         <v>46162.55853556713</v>
       </c>
-      <c r="C70" s="6"/>
+      <c r="C70" s="5">
+        <v>46247.81526716435</v>
+      </c>
       <c r="D70" s="5">
-        <v>46225.81140046296</v>
+        <v>46247.81528174768</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>227</v>
@@ -6210,8 +6242,12 @@
       <c r="Q70" s="6"/>
       <c r="R70" s="6"/>
       <c r="S70" s="6"/>
-      <c r="T70" s="6"/>
-      <c r="U70" s="6"/>
+      <c r="T70" s="6">
+        <v>1</v>
+      </c>
+      <c r="U70" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
@@ -6945,9 +6981,11 @@
       <c r="B84" s="5">
         <v>46162.55862063657</v>
       </c>
-      <c r="C84" s="6"/>
+      <c r="C84" s="5">
+        <v>46247.81329474537</v>
+      </c>
       <c r="D84" s="5">
-        <v>46225.81192504629</v>
+        <v>46247.813307812496</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>254</v>
@@ -6995,10 +7033,10 @@
         <v>33</v>
       </c>
       <c r="T84" s="6">
-        <v>0</v>
-      </c>
-      <c r="U84" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U84" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
@@ -7008,9 +7046,11 @@
       <c r="B85" s="9">
         <v>46162.558626620375</v>
       </c>
-      <c r="C85" s="10"/>
+      <c r="C85" s="9">
+        <v>46247.81326572917</v>
+      </c>
       <c r="D85" s="9">
-        <v>46225.81138908565</v>
+        <v>46247.813273101856</v>
       </c>
       <c r="E85" s="10" t="s">
         <v>190</v>
@@ -7061,9 +7101,11 @@
       <c r="B86" s="5">
         <v>46162.55863280092</v>
       </c>
-      <c r="C86" s="6"/>
+      <c r="C86" s="5">
+        <v>46247.81326645833</v>
+      </c>
       <c r="D86" s="5">
-        <v>46225.81137782407</v>
+        <v>46247.81327356481</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>190</v>
@@ -7114,9 +7156,11 @@
       <c r="B87" s="9">
         <v>46162.55863850695</v>
       </c>
-      <c r="C87" s="10"/>
+      <c r="C87" s="9">
+        <v>46247.81326702546</v>
+      </c>
       <c r="D87" s="9">
-        <v>46225.81136515047</v>
+        <v>46247.813274050925</v>
       </c>
       <c r="E87" s="10" t="s">
         <v>190</v>
@@ -7167,9 +7211,11 @@
       <c r="B88" s="5">
         <v>46162.558644247685</v>
       </c>
-      <c r="C88" s="6"/>
+      <c r="C88" s="5">
+        <v>46247.81326759259</v>
+      </c>
       <c r="D88" s="5">
-        <v>46225.811345740745</v>
+        <v>46247.81327449074</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>190</v>
@@ -7220,9 +7266,11 @@
       <c r="B89" s="9">
         <v>46162.55864990741</v>
       </c>
-      <c r="C89" s="10"/>
+      <c r="C89" s="9">
+        <v>46247.81326810185</v>
+      </c>
       <c r="D89" s="9">
-        <v>46225.811355625</v>
+        <v>46247.81327490741</v>
       </c>
       <c r="E89" s="10" t="s">
         <v>196</v>
@@ -7273,9 +7321,11 @@
       <c r="B90" s="5">
         <v>46162.56148016204</v>
       </c>
-      <c r="C90" s="6"/>
+      <c r="C90" s="5">
+        <v>46247.813268680555</v>
+      </c>
       <c r="D90" s="5">
-        <v>46225.81132334491</v>
+        <v>46247.81327533565</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>196</v>
@@ -7326,9 +7376,11 @@
       <c r="B91" s="9">
         <v>46162.561489201384</v>
       </c>
-      <c r="C91" s="10"/>
+      <c r="C91" s="9">
+        <v>46247.81326920139</v>
+      </c>
       <c r="D91" s="9">
-        <v>46225.81131275463</v>
+        <v>46247.81327569444</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>196</v>
@@ -7379,9 +7431,11 @@
       <c r="B92" s="5">
         <v>46162.56149930556</v>
       </c>
-      <c r="C92" s="6"/>
+      <c r="C92" s="5">
+        <v>46247.813269606486</v>
+      </c>
       <c r="D92" s="5">
-        <v>46225.81130295139</v>
+        <v>46247.81327605324</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>196</v>
@@ -7432,9 +7486,11 @@
       <c r="B93" s="9">
         <v>46162.561507199076</v>
       </c>
-      <c r="C93" s="10"/>
+      <c r="C93" s="9">
+        <v>46247.81327021991</v>
+      </c>
       <c r="D93" s="9">
-        <v>46225.81129587963</v>
+        <v>46247.81327640046</v>
       </c>
       <c r="E93" s="10" t="s">
         <v>196</v>
@@ -7485,9 +7541,11 @@
       <c r="B94" s="5">
         <v>46162.56151613426</v>
       </c>
-      <c r="C94" s="6"/>
+      <c r="C94" s="5">
+        <v>46247.813270729166</v>
+      </c>
       <c r="D94" s="5">
-        <v>46225.81128686343</v>
+        <v>46247.813276747685</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>196</v>
@@ -7538,9 +7596,11 @@
       <c r="B95" s="9">
         <v>46162.56152413195</v>
       </c>
-      <c r="C95" s="10"/>
+      <c r="C95" s="9">
+        <v>46247.81327126158</v>
+      </c>
       <c r="D95" s="9">
-        <v>46225.81127690972</v>
+        <v>46247.81327708333</v>
       </c>
       <c r="E95" s="10" t="s">
         <v>196</v>
@@ -7591,9 +7651,11 @@
       <c r="B96" s="5">
         <v>46162.56153119213</v>
       </c>
-      <c r="C96" s="6"/>
+      <c r="C96" s="5">
+        <v>46247.813271747684</v>
+      </c>
       <c r="D96" s="5">
-        <v>46225.81127016204</v>
+        <v>46247.81327741898</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>196</v>
@@ -7644,9 +7706,11 @@
       <c r="B97" s="9">
         <v>46162.55865439815</v>
       </c>
-      <c r="C97" s="10"/>
+      <c r="C97" s="9">
+        <v>46247.81345563657</v>
+      </c>
       <c r="D97" s="9">
-        <v>46218.20591833333</v>
+        <v>46247.815585648146</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>273</v>
@@ -7655,10 +7719,10 @@
         <v>26</v>
       </c>
       <c r="G97" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H97" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="H97" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="I97" s="9">
         <v>46217</v>
@@ -7694,10 +7758,10 @@
         <v>33</v>
       </c>
       <c r="T97" s="10">
-        <v>0</v>
-      </c>
-      <c r="U97" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U97" s="12" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
@@ -7707,9 +7771,11 @@
       <c r="B98" s="5">
         <v>46162.55865909722</v>
       </c>
-      <c r="C98" s="6"/>
+      <c r="C98" s="5">
+        <v>46247.81341994213</v>
+      </c>
       <c r="D98" s="5">
-        <v>46217.16848263889</v>
+        <v>46247.81342832176</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>190</v>
@@ -7718,10 +7784,10 @@
         <v>26</v>
       </c>
       <c r="G98" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="H98" s="6" t="s">
         <v>158</v>
-      </c>
-      <c r="H98" s="6" t="s">
-        <v>159</v>
       </c>
       <c r="I98" s="5">
         <v>46217</v>
@@ -7760,9 +7826,11 @@
       <c r="B99" s="9">
         <v>46162.55866501157</v>
       </c>
-      <c r="C99" s="10"/>
+      <c r="C99" s="9">
+        <v>46247.81342078703</v>
+      </c>
       <c r="D99" s="9">
-        <v>46217.168484050926</v>
+        <v>46247.813428761576</v>
       </c>
       <c r="E99" s="10" t="s">
         <v>190</v>
@@ -7771,10 +7839,10 @@
         <v>26</v>
       </c>
       <c r="G99" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H99" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="H99" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="I99" s="9">
         <v>46217</v>
@@ -7813,9 +7881,11 @@
       <c r="B100" s="5">
         <v>46162.55867084491</v>
       </c>
-      <c r="C100" s="6"/>
+      <c r="C100" s="5">
+        <v>46247.81342143519</v>
+      </c>
       <c r="D100" s="5">
-        <v>46217.16847319444</v>
+        <v>46247.81342914352</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>190</v>
@@ -7824,10 +7894,10 @@
         <v>26</v>
       </c>
       <c r="G100" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="H100" s="6" t="s">
         <v>158</v>
-      </c>
-      <c r="H100" s="6" t="s">
-        <v>159</v>
       </c>
       <c r="I100" s="5">
         <v>46217</v>
@@ -7866,9 +7936,11 @@
       <c r="B101" s="9">
         <v>46162.558676597226</v>
       </c>
-      <c r="C101" s="10"/>
+      <c r="C101" s="9">
+        <v>46247.81342208333</v>
+      </c>
       <c r="D101" s="9">
-        <v>46217.16847716435</v>
+        <v>46247.813429490736</v>
       </c>
       <c r="E101" s="10" t="s">
         <v>190</v>
@@ -7877,10 +7949,10 @@
         <v>26</v>
       </c>
       <c r="G101" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H101" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="H101" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="I101" s="9">
         <v>46217</v>
@@ -7919,9 +7991,11 @@
       <c r="B102" s="5">
         <v>46162.55868239583</v>
       </c>
-      <c r="C102" s="6"/>
+      <c r="C102" s="5">
+        <v>46247.81342266204</v>
+      </c>
       <c r="D102" s="5">
-        <v>46217.168485312504</v>
+        <v>46247.81342986111</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>196</v>
@@ -7930,10 +8004,10 @@
         <v>26</v>
       </c>
       <c r="G102" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="H102" s="6" t="s">
         <v>158</v>
-      </c>
-      <c r="H102" s="6" t="s">
-        <v>159</v>
       </c>
       <c r="I102" s="5">
         <v>46217</v>
@@ -7972,9 +8046,11 @@
       <c r="B103" s="9">
         <v>46162.56176834491</v>
       </c>
-      <c r="C103" s="10"/>
+      <c r="C103" s="9">
+        <v>46247.81342333333</v>
+      </c>
       <c r="D103" s="9">
-        <v>46217.16846244213</v>
+        <v>46247.813430208334</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>196</v>
@@ -7983,10 +8059,10 @@
         <v>26</v>
       </c>
       <c r="G103" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H103" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="H103" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="I103" s="9">
         <v>46217</v>
@@ -8025,9 +8101,11 @@
       <c r="B104" s="5">
         <v>46162.56177670139</v>
       </c>
-      <c r="C104" s="6"/>
+      <c r="C104" s="5">
+        <v>46247.813423935186</v>
+      </c>
       <c r="D104" s="5">
-        <v>46224.87647666667</v>
+        <v>46247.81343056713</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>196</v>
@@ -8036,10 +8114,10 @@
         <v>26</v>
       </c>
       <c r="G104" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="H104" s="6" t="s">
         <v>158</v>
-      </c>
-      <c r="H104" s="6" t="s">
-        <v>159</v>
       </c>
       <c r="I104" s="5">
         <v>46217</v>
@@ -8078,9 +8156,11 @@
       <c r="B105" s="9">
         <v>46162.56178474537</v>
       </c>
-      <c r="C105" s="10"/>
+      <c r="C105" s="9">
+        <v>46247.81342449074</v>
+      </c>
       <c r="D105" s="9">
-        <v>46217.16846583333</v>
+        <v>46247.81343096065</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>196</v>
@@ -8089,10 +8169,10 @@
         <v>26</v>
       </c>
       <c r="G105" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H105" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="H105" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="I105" s="9">
         <v>46217</v>
@@ -8131,9 +8211,11 @@
       <c r="B106" s="5">
         <v>46162.56179298611</v>
       </c>
-      <c r="C106" s="6"/>
+      <c r="C106" s="5">
+        <v>46247.8134250463</v>
+      </c>
       <c r="D106" s="5">
-        <v>46217.16846726852</v>
+        <v>46247.813431284725</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>196</v>
@@ -8142,10 +8224,10 @@
         <v>26</v>
       </c>
       <c r="G106" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="H106" s="6" t="s">
         <v>158</v>
-      </c>
-      <c r="H106" s="6" t="s">
-        <v>159</v>
       </c>
       <c r="I106" s="5">
         <v>46217</v>
@@ -8184,9 +8266,11 @@
       <c r="B107" s="9">
         <v>46162.5618009375</v>
       </c>
-      <c r="C107" s="10"/>
+      <c r="C107" s="9">
+        <v>46247.813425636574</v>
+      </c>
       <c r="D107" s="9">
-        <v>46217.16846878472</v>
+        <v>46247.81343163195</v>
       </c>
       <c r="E107" s="10" t="s">
         <v>196</v>
@@ -8195,10 +8279,10 @@
         <v>26</v>
       </c>
       <c r="G107" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H107" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="H107" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="I107" s="9">
         <v>46217</v>
@@ -8237,9 +8321,11 @@
       <c r="B108" s="5">
         <v>46162.56180909723</v>
       </c>
-      <c r="C108" s="6"/>
+      <c r="C108" s="5">
+        <v>46247.8134262963</v>
+      </c>
       <c r="D108" s="5">
-        <v>46217.168470358796</v>
+        <v>46247.81343196759</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>196</v>
@@ -8248,10 +8334,10 @@
         <v>26</v>
       </c>
       <c r="G108" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="H108" s="6" t="s">
         <v>158</v>
-      </c>
-      <c r="H108" s="6" t="s">
-        <v>159</v>
       </c>
       <c r="I108" s="5">
         <v>46217</v>
@@ -8290,9 +8376,11 @@
       <c r="B109" s="9">
         <v>46162.56181716435</v>
       </c>
-      <c r="C109" s="10"/>
+      <c r="C109" s="9">
+        <v>46247.81342679398</v>
+      </c>
       <c r="D109" s="9">
-        <v>46217.16847178241</v>
+        <v>46247.81343231481</v>
       </c>
       <c r="E109" s="10" t="s">
         <v>196</v>
@@ -8301,10 +8389,10 @@
         <v>26</v>
       </c>
       <c r="G109" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H109" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="H109" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="I109" s="9">
         <v>46217</v>
@@ -8433,7 +8521,7 @@
         <v>205</v>
       </c>
       <c r="O111" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P111" s="10" t="s">
         <v>297</v>
@@ -8498,7 +8586,7 @@
         <v>205</v>
       </c>
       <c r="O112" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="P112" s="6" t="s">
         <v>300</v>
@@ -8563,7 +8651,7 @@
         <v>205</v>
       </c>
       <c r="O113" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P113" s="10" t="s">
         <v>303</v>
@@ -8628,7 +8716,7 @@
         <v>205</v>
       </c>
       <c r="O114" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P114" s="6" t="s">
         <v>306</v>
@@ -8658,7 +8746,7 @@
       </c>
       <c r="C115" s="10"/>
       <c r="D115" s="9">
-        <v>46162.64775322917</v>
+        <v>46247.81444270833</v>
       </c>
       <c r="E115" s="10" t="s">
         <v>308</v>
@@ -8703,9 +8791,11 @@
       <c r="B116" s="5">
         <v>46162.55872223379</v>
       </c>
-      <c r="C116" s="6"/>
+      <c r="C116" s="5">
+        <v>46247.813576307875</v>
+      </c>
       <c r="D116" s="5">
-        <v>46237.54090622685</v>
+        <v>46247.815586412034</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>311</v>
@@ -8753,10 +8843,10 @@
         <v>33</v>
       </c>
       <c r="T116" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U116" s="12" t="s">
-        <v>93</v>
+        <v>188</v>
       </c>
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
@@ -8766,9 +8856,11 @@
       <c r="B117" s="9">
         <v>46162.55873068287</v>
       </c>
-      <c r="C117" s="10"/>
+      <c r="C117" s="9">
+        <v>46247.813550949075</v>
+      </c>
       <c r="D117" s="9">
-        <v>46224.25040153935</v>
+        <v>46247.8155793287</v>
       </c>
       <c r="E117" s="10" t="s">
         <v>190</v>
@@ -8819,9 +8911,11 @@
       <c r="B118" s="5">
         <v>46162.558735011575</v>
       </c>
-      <c r="C118" s="6"/>
+      <c r="C118" s="5">
+        <v>46247.81355158565</v>
+      </c>
       <c r="D118" s="5">
-        <v>46224.25040292824</v>
+        <v>46247.81355893519</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>190</v>
@@ -8872,9 +8966,11 @@
       <c r="B119" s="9">
         <v>46162.55873951389</v>
       </c>
-      <c r="C119" s="10"/>
+      <c r="C119" s="9">
+        <v>46247.81355201389</v>
+      </c>
       <c r="D119" s="9">
-        <v>46224.25044962963</v>
+        <v>46247.81355928241</v>
       </c>
       <c r="E119" s="10" t="s">
         <v>190</v>
@@ -8925,9 +9021,11 @@
       <c r="B120" s="5">
         <v>46162.55874386574</v>
       </c>
-      <c r="C120" s="6"/>
+      <c r="C120" s="5">
+        <v>46247.813552638894</v>
+      </c>
       <c r="D120" s="5">
-        <v>46224.25045101852</v>
+        <v>46247.81355965278</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>190</v>
@@ -8978,9 +9076,11 @@
       <c r="B121" s="9">
         <v>46162.55874813657</v>
       </c>
-      <c r="C121" s="10"/>
+      <c r="C121" s="9">
+        <v>46247.813553252316</v>
+      </c>
       <c r="D121" s="9">
-        <v>46224.25040421296</v>
+        <v>46247.813559988426</v>
       </c>
       <c r="E121" s="10" t="s">
         <v>196</v>
@@ -9031,9 +9131,11 @@
       <c r="B122" s="5">
         <v>46162.56516702546</v>
       </c>
-      <c r="C122" s="6"/>
+      <c r="C122" s="5">
+        <v>46247.81355381945</v>
+      </c>
       <c r="D122" s="5">
-        <v>46224.25042715278</v>
+        <v>46247.81356034722</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>196</v>
@@ -9084,9 +9186,11 @@
       <c r="B123" s="9">
         <v>46162.56517383102</v>
       </c>
-      <c r="C123" s="10"/>
+      <c r="C123" s="9">
+        <v>46247.813554374996</v>
+      </c>
       <c r="D123" s="9">
-        <v>46224.2504290625</v>
+        <v>46247.813560740746</v>
       </c>
       <c r="E123" s="10" t="s">
         <v>196</v>
@@ -9137,9 +9241,11 @@
       <c r="B124" s="5">
         <v>46162.565181134254</v>
       </c>
-      <c r="C124" s="6"/>
+      <c r="C124" s="5">
+        <v>46247.81355496528</v>
+      </c>
       <c r="D124" s="5">
-        <v>46224.250430555556</v>
+        <v>46247.81356108796</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>196</v>
@@ -9190,9 +9296,11 @@
       <c r="B125" s="9">
         <v>46162.565189201385</v>
       </c>
-      <c r="C125" s="10"/>
+      <c r="C125" s="9">
+        <v>46247.81355553241</v>
+      </c>
       <c r="D125" s="9">
-        <v>46224.25043193287</v>
+        <v>46247.813561435185</v>
       </c>
       <c r="E125" s="10" t="s">
         <v>196</v>
@@ -9243,9 +9351,11 @@
       <c r="B126" s="5">
         <v>46162.56519680556</v>
       </c>
-      <c r="C126" s="6"/>
+      <c r="C126" s="5">
+        <v>46247.81355611111</v>
+      </c>
       <c r="D126" s="5">
-        <v>46224.250433402776</v>
+        <v>46247.81356178241</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>196</v>
@@ -9296,9 +9406,11 @@
       <c r="B127" s="9">
         <v>46162.565205590276</v>
       </c>
-      <c r="C127" s="10"/>
+      <c r="C127" s="9">
+        <v>46247.81355662037</v>
+      </c>
       <c r="D127" s="9">
-        <v>46224.25043480324</v>
+        <v>46247.813562129624</v>
       </c>
       <c r="E127" s="10" t="s">
         <v>196</v>
@@ -9349,9 +9461,11 @@
       <c r="B128" s="5">
         <v>46162.565212013884</v>
       </c>
-      <c r="C128" s="6"/>
+      <c r="C128" s="5">
+        <v>46247.81355717593</v>
+      </c>
       <c r="D128" s="5">
-        <v>46224.25043630787</v>
+        <v>46247.81356247685</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>196</v>
@@ -9402,9 +9516,11 @@
       <c r="B129" s="9">
         <v>46162.558751550925</v>
       </c>
-      <c r="C129" s="10"/>
+      <c r="C129" s="9">
+        <v>46247.81391107639</v>
+      </c>
       <c r="D129" s="9">
-        <v>46237.54094651621</v>
+        <v>46247.81393420139</v>
       </c>
       <c r="E129" s="10" t="s">
         <v>328</v>
@@ -9452,7 +9568,7 @@
         <v>33</v>
       </c>
       <c r="T129" s="10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U129" s="7" t="s">
         <v>27</v>
@@ -9465,9 +9581,11 @@
       <c r="B130" s="5">
         <v>46162.558756238424</v>
       </c>
-      <c r="C130" s="6"/>
+      <c r="C130" s="5">
+        <v>46247.81387784722</v>
+      </c>
       <c r="D130" s="5">
-        <v>46223.57901649305</v>
+        <v>46247.81388666667</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>190</v>
@@ -9516,9 +9634,11 @@
       <c r="B131" s="9">
         <v>46162.55876204861</v>
       </c>
-      <c r="C131" s="10"/>
+      <c r="C131" s="9">
+        <v>46247.813878773144</v>
+      </c>
       <c r="D131" s="9">
-        <v>46223.57901584491</v>
+        <v>46247.81388728009</v>
       </c>
       <c r="E131" s="10" t="s">
         <v>190</v>
@@ -9567,9 +9687,11 @@
       <c r="B132" s="5">
         <v>46162.55876745371</v>
       </c>
-      <c r="C132" s="6"/>
+      <c r="C132" s="5">
+        <v>46247.81387945602</v>
+      </c>
       <c r="D132" s="5">
-        <v>46223.57901519676</v>
+        <v>46247.81388778935</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>190</v>
@@ -9618,9 +9740,11 @@
       <c r="B133" s="9">
         <v>46162.558773888886</v>
       </c>
-      <c r="C133" s="10"/>
+      <c r="C133" s="9">
+        <v>46247.813880104164</v>
+      </c>
       <c r="D133" s="9">
-        <v>46223.57901452546</v>
+        <v>46247.81388819445</v>
       </c>
       <c r="E133" s="10" t="s">
         <v>190</v>
@@ -9669,9 +9793,11 @@
       <c r="B134" s="5">
         <v>46162.558827430556</v>
       </c>
-      <c r="C134" s="6"/>
+      <c r="C134" s="5">
+        <v>46247.81388079861</v>
+      </c>
       <c r="D134" s="5">
-        <v>46223.579013888884</v>
+        <v>46247.81388861111</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>196</v>
@@ -9720,9 +9846,11 @@
       <c r="B135" s="9">
         <v>46162.565477233795</v>
       </c>
-      <c r="C135" s="10"/>
+      <c r="C135" s="9">
+        <v>46247.81388153935</v>
+      </c>
       <c r="D135" s="9">
-        <v>46223.579013229166</v>
+        <v>46247.81388916667</v>
       </c>
       <c r="E135" s="10" t="s">
         <v>196</v>
@@ -9771,9 +9899,11 @@
       <c r="B136" s="5">
         <v>46162.56548539352</v>
       </c>
-      <c r="C136" s="6"/>
+      <c r="C136" s="5">
+        <v>46247.81388210648</v>
+      </c>
       <c r="D136" s="5">
-        <v>46223.579012546295</v>
+        <v>46247.81388960648</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>196</v>
@@ -9822,9 +9952,11 @@
       <c r="B137" s="9">
         <v>46162.56549420139</v>
       </c>
-      <c r="C137" s="10"/>
+      <c r="C137" s="9">
+        <v>46247.81388266204</v>
+      </c>
       <c r="D137" s="9">
-        <v>46223.579011875</v>
+        <v>46247.81389002315</v>
       </c>
       <c r="E137" s="10" t="s">
         <v>196</v>
@@ -9873,9 +10005,11 @@
       <c r="B138" s="5">
         <v>46162.56549981482</v>
       </c>
-      <c r="C138" s="6"/>
+      <c r="C138" s="5">
+        <v>46247.81388327546</v>
+      </c>
       <c r="D138" s="5">
-        <v>46223.57901104167</v>
+        <v>46247.81389039352</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>196</v>
@@ -9924,9 +10058,11 @@
       <c r="B139" s="9">
         <v>46162.565507719904</v>
       </c>
-      <c r="C139" s="10"/>
+      <c r="C139" s="9">
+        <v>46247.813883842595</v>
+      </c>
       <c r="D139" s="9">
-        <v>46223.57901035879</v>
+        <v>46247.81389078704</v>
       </c>
       <c r="E139" s="10" t="s">
         <v>196</v>
@@ -9975,9 +10111,11 @@
       <c r="B140" s="5">
         <v>46162.56551637732</v>
       </c>
-      <c r="C140" s="6"/>
+      <c r="C140" s="5">
+        <v>46247.813884421295</v>
+      </c>
       <c r="D140" s="5">
-        <v>46223.579009733796</v>
+        <v>46247.813891157406</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>196</v>
@@ -10026,9 +10164,11 @@
       <c r="B141" s="9">
         <v>46162.56598206019</v>
       </c>
-      <c r="C141" s="10"/>
+      <c r="C141" s="9">
+        <v>46247.8138850463</v>
+      </c>
       <c r="D141" s="9">
-        <v>46223.57900907408</v>
+        <v>46247.81389152778</v>
       </c>
       <c r="E141" s="10" t="s">
         <v>196</v>
@@ -10077,9 +10217,11 @@
       <c r="B142" s="5">
         <v>46162.55883354167</v>
       </c>
-      <c r="C142" s="6"/>
+      <c r="C142" s="5">
+        <v>46247.814077731484</v>
+      </c>
       <c r="D142" s="5">
-        <v>46223.57990805556</v>
+        <v>46247.81409195602</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>352</v>
@@ -10127,10 +10269,10 @@
         <v>33</v>
       </c>
       <c r="T142" s="6">
-        <v>0</v>
-      </c>
-      <c r="U142" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U142" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
@@ -10140,9 +10282,11 @@
       <c r="B143" s="9">
         <v>46162.55883898148</v>
       </c>
-      <c r="C143" s="10"/>
+      <c r="C143" s="9">
+        <v>46247.81404020834</v>
+      </c>
       <c r="D143" s="9">
-        <v>46223.57929469907</v>
+        <v>46247.81405185185</v>
       </c>
       <c r="E143" s="10" t="s">
         <v>190</v>
@@ -10193,9 +10337,11 @@
       <c r="B144" s="5">
         <v>46162.55884618056</v>
       </c>
-      <c r="C144" s="6"/>
+      <c r="C144" s="5">
+        <v>46247.81404131945</v>
+      </c>
       <c r="D144" s="5">
-        <v>46223.57929405093</v>
+        <v>46247.81405244213</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>190</v>
@@ -10246,9 +10392,11 @@
       <c r="B145" s="9">
         <v>46162.55885335648</v>
       </c>
-      <c r="C145" s="10"/>
+      <c r="C145" s="9">
+        <v>46247.814042314814</v>
+      </c>
       <c r="D145" s="9">
-        <v>46223.5792933912</v>
+        <v>46247.81405292824</v>
       </c>
       <c r="E145" s="10" t="s">
         <v>190</v>
@@ -10299,9 +10447,11 @@
       <c r="B146" s="5">
         <v>46162.558860624995</v>
       </c>
-      <c r="C146" s="6"/>
+      <c r="C146" s="5">
+        <v>46247.81404347222</v>
+      </c>
       <c r="D146" s="5">
-        <v>46223.579292766204</v>
+        <v>46247.814053379625</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>190</v>
@@ -10352,9 +10502,11 @@
       <c r="B147" s="9">
         <v>46162.558867395834</v>
       </c>
-      <c r="C147" s="10"/>
+      <c r="C147" s="9">
+        <v>46247.81404434028</v>
+      </c>
       <c r="D147" s="9">
-        <v>46223.57929214121</v>
+        <v>46247.81405421296</v>
       </c>
       <c r="E147" s="10" t="s">
         <v>196</v>
@@ -10405,9 +10557,11 @@
       <c r="B148" s="5">
         <v>46162.566146365745</v>
       </c>
-      <c r="C148" s="6"/>
+      <c r="C148" s="5">
+        <v>46247.81404521991</v>
+      </c>
       <c r="D148" s="5">
-        <v>46223.5792915162</v>
+        <v>46247.814054664355</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>196</v>
@@ -10458,9 +10612,11 @@
       <c r="B149" s="9">
         <v>46162.566153101856</v>
       </c>
-      <c r="C149" s="10"/>
+      <c r="C149" s="9">
+        <v>46247.814045949075</v>
+      </c>
       <c r="D149" s="9">
-        <v>46223.57929087963</v>
+        <v>46247.81405508102</v>
       </c>
       <c r="E149" s="10" t="s">
         <v>196</v>
@@ -10511,9 +10667,11 @@
       <c r="B150" s="5">
         <v>46162.56617111111</v>
       </c>
-      <c r="C150" s="6"/>
+      <c r="C150" s="5">
+        <v>46247.81404670139</v>
+      </c>
       <c r="D150" s="5">
-        <v>46223.57929026621</v>
+        <v>46247.814055509254</v>
       </c>
       <c r="E150" s="6" t="s">
         <v>196</v>
@@ -10564,9 +10722,11 @@
       <c r="B151" s="9">
         <v>46162.56618105324</v>
       </c>
-      <c r="C151" s="10"/>
+      <c r="C151" s="9">
+        <v>46247.81404748843</v>
+      </c>
       <c r="D151" s="9">
-        <v>46223.57928965278</v>
+        <v>46247.81405601852</v>
       </c>
       <c r="E151" s="10" t="s">
         <v>346</v>
@@ -10617,9 +10777,11 @@
       <c r="B152" s="5">
         <v>46162.56618987268</v>
       </c>
-      <c r="C152" s="6"/>
+      <c r="C152" s="5">
+        <v>46247.814048263885</v>
+      </c>
       <c r="D152" s="5">
-        <v>46223.57928883102</v>
+        <v>46247.81405644676</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>196</v>
@@ -10670,9 +10832,11 @@
       <c r="B153" s="9">
         <v>46162.56620271991</v>
       </c>
-      <c r="C153" s="10"/>
+      <c r="C153" s="9">
+        <v>46247.81404895833</v>
+      </c>
       <c r="D153" s="9">
-        <v>46223.57928822917</v>
+        <v>46247.81405685185</v>
       </c>
       <c r="E153" s="10" t="s">
         <v>196</v>
@@ -10723,9 +10887,11 @@
       <c r="B154" s="5">
         <v>46162.56620673611</v>
       </c>
-      <c r="C154" s="6"/>
+      <c r="C154" s="5">
+        <v>46247.81404971065</v>
+      </c>
       <c r="D154" s="5">
-        <v>46223.579287615736</v>
+        <v>46247.81405725694</v>
       </c>
       <c r="E154" s="6" t="s">
         <v>196</v>
@@ -10776,9 +10942,11 @@
       <c r="B155" s="9">
         <v>46162.558871574074</v>
       </c>
-      <c r="C155" s="10"/>
+      <c r="C155" s="9">
+        <v>46247.814219699074</v>
+      </c>
       <c r="D155" s="9">
-        <v>46224.18423814815</v>
+        <v>46247.814231689816</v>
       </c>
       <c r="E155" s="10" t="s">
         <v>372</v>
@@ -10826,10 +10994,10 @@
         <v>33</v>
       </c>
       <c r="T155" s="10">
-        <v>0</v>
-      </c>
-      <c r="U155" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U155" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="156" spans="1:21" x14ac:dyDescent="0.25">
@@ -10839,9 +11007,11 @@
       <c r="B156" s="5">
         <v>46162.55887622685</v>
       </c>
-      <c r="C156" s="6"/>
+      <c r="C156" s="5">
+        <v>46247.81418356481</v>
+      </c>
       <c r="D156" s="5">
-        <v>46225.87106959491</v>
+        <v>46247.81419292824</v>
       </c>
       <c r="E156" s="6" t="s">
         <v>190</v>
@@ -10892,9 +11062,11 @@
       <c r="B157" s="9">
         <v>46162.55888300926</v>
       </c>
-      <c r="C157" s="10"/>
+      <c r="C157" s="9">
+        <v>46247.814184456016</v>
+      </c>
       <c r="D157" s="9">
-        <v>46225.87107101852</v>
+        <v>46247.81419348379</v>
       </c>
       <c r="E157" s="10" t="s">
         <v>190</v>
@@ -10945,9 +11117,11 @@
       <c r="B158" s="5">
         <v>46162.558892581015</v>
       </c>
-      <c r="C158" s="6"/>
+      <c r="C158" s="5">
+        <v>46247.814185104166</v>
+      </c>
       <c r="D158" s="5">
-        <v>46225.87107528935</v>
+        <v>46247.81419395833</v>
       </c>
       <c r="E158" s="6" t="s">
         <v>190</v>
@@ -10998,9 +11172,11 @@
       <c r="B159" s="9">
         <v>46162.55889858796</v>
       </c>
-      <c r="C159" s="10"/>
+      <c r="C159" s="9">
+        <v>46247.81418613426</v>
+      </c>
       <c r="D159" s="9">
-        <v>46225.87107458334</v>
+        <v>46247.814194398146</v>
       </c>
       <c r="E159" s="10" t="s">
         <v>190</v>
@@ -11051,9 +11227,11 @@
       <c r="B160" s="5">
         <v>46162.558904618054</v>
       </c>
-      <c r="C160" s="6"/>
+      <c r="C160" s="5">
+        <v>46247.81418677083</v>
+      </c>
       <c r="D160" s="5">
-        <v>46223.57947667824</v>
+        <v>46247.81419479167</v>
       </c>
       <c r="E160" s="6" t="s">
         <v>196</v>
@@ -11104,9 +11282,11 @@
       <c r="B161" s="9">
         <v>46162.566379375</v>
       </c>
-      <c r="C161" s="10"/>
+      <c r="C161" s="9">
+        <v>46247.81418747685</v>
+      </c>
       <c r="D161" s="9">
-        <v>46225.87106449074</v>
+        <v>46247.81419527778</v>
       </c>
       <c r="E161" s="10" t="s">
         <v>196</v>
@@ -11157,9 +11337,11 @@
       <c r="B162" s="5">
         <v>46162.56638695602</v>
       </c>
-      <c r="C162" s="6"/>
+      <c r="C162" s="5">
+        <v>46247.81418810185</v>
+      </c>
       <c r="D162" s="5">
-        <v>46225.87106525463</v>
+        <v>46247.814195659725</v>
       </c>
       <c r="E162" s="6" t="s">
         <v>196</v>
@@ -11210,9 +11392,11 @@
       <c r="B163" s="9">
         <v>46162.56639532407</v>
       </c>
-      <c r="C163" s="10"/>
+      <c r="C163" s="9">
+        <v>46247.814188749995</v>
+      </c>
       <c r="D163" s="9">
-        <v>46225.871065949075</v>
+        <v>46247.81419597223</v>
       </c>
       <c r="E163" s="10" t="s">
         <v>196</v>
@@ -11263,9 +11447,11 @@
       <c r="B164" s="5">
         <v>46162.56640418981</v>
       </c>
-      <c r="C164" s="6"/>
+      <c r="C164" s="5">
+        <v>46247.81418947916</v>
+      </c>
       <c r="D164" s="5">
-        <v>46225.8710666088</v>
+        <v>46247.81419634259</v>
       </c>
       <c r="E164" s="6" t="s">
         <v>196</v>
@@ -11316,9 +11502,11 @@
       <c r="B165" s="9">
         <v>46162.56641240741</v>
       </c>
-      <c r="C165" s="10"/>
+      <c r="C165" s="9">
+        <v>46247.81419010417</v>
+      </c>
       <c r="D165" s="9">
-        <v>46225.87106722222</v>
+        <v>46247.81419680556</v>
       </c>
       <c r="E165" s="10" t="s">
         <v>196</v>
@@ -11369,9 +11557,11 @@
       <c r="B166" s="5">
         <v>46162.56642033564</v>
       </c>
-      <c r="C166" s="6"/>
+      <c r="C166" s="5">
+        <v>46247.81419077546</v>
+      </c>
       <c r="D166" s="5">
-        <v>46225.87106789352</v>
+        <v>46247.8141971875</v>
       </c>
       <c r="E166" s="6" t="s">
         <v>196</v>
@@ -11422,9 +11612,11 @@
       <c r="B167" s="9">
         <v>46162.566427708334</v>
       </c>
-      <c r="C167" s="10"/>
+      <c r="C167" s="9">
+        <v>46247.81419138889</v>
+      </c>
       <c r="D167" s="9">
-        <v>46225.87106853009</v>
+        <v>46247.814197569445</v>
       </c>
       <c r="E167" s="10" t="s">
         <v>196</v>
@@ -11475,9 +11667,11 @@
       <c r="B168" s="5">
         <v>46162.558908946754</v>
       </c>
-      <c r="C168" s="6"/>
+      <c r="C168" s="5">
+        <v>46247.81443539352</v>
+      </c>
       <c r="D168" s="5">
-        <v>46225.18524023148</v>
+        <v>46247.814451053244</v>
       </c>
       <c r="E168" s="6" t="s">
         <v>397</v>
@@ -11525,10 +11719,10 @@
         <v>33</v>
       </c>
       <c r="T168" s="6">
-        <v>0</v>
-      </c>
-      <c r="U168" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U168" s="12" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="169" spans="1:21" x14ac:dyDescent="0.25">
@@ -11538,9 +11732,11 @@
       <c r="B169" s="9">
         <v>46162.55891369213</v>
       </c>
-      <c r="C169" s="10"/>
+      <c r="C169" s="9">
+        <v>46247.81438027778</v>
+      </c>
       <c r="D169" s="9">
-        <v>46224.25045532407</v>
+        <v>46247.81440623842</v>
       </c>
       <c r="E169" s="10" t="s">
         <v>190</v>
@@ -11589,9 +11785,11 @@
       <c r="B170" s="5">
         <v>46162.55891930556</v>
       </c>
-      <c r="C170" s="6"/>
+      <c r="C170" s="5">
+        <v>46247.81438157408</v>
+      </c>
       <c r="D170" s="5">
-        <v>46224.25039887731</v>
+        <v>46247.814408680555</v>
       </c>
       <c r="E170" s="6" t="s">
         <v>190</v>
@@ -11640,9 +11838,11 @@
       <c r="B171" s="9">
         <v>46162.558924930556</v>
       </c>
-      <c r="C171" s="10"/>
+      <c r="C171" s="9">
+        <v>46247.81438563658</v>
+      </c>
       <c r="D171" s="9">
-        <v>46224.250400185185</v>
+        <v>46247.81441115741</v>
       </c>
       <c r="E171" s="10" t="s">
         <v>190</v>
@@ -11691,9 +11891,11 @@
       <c r="B172" s="5">
         <v>46162.55893104167</v>
       </c>
-      <c r="C172" s="6"/>
+      <c r="C172" s="5">
+        <v>46247.81438819444</v>
+      </c>
       <c r="D172" s="5">
-        <v>46224.25039688658</v>
+        <v>46247.814413726854</v>
       </c>
       <c r="E172" s="6" t="s">
         <v>190</v>
@@ -11742,9 +11944,11 @@
       <c r="B173" s="9">
         <v>46162.55893646991</v>
       </c>
-      <c r="C173" s="10"/>
+      <c r="C173" s="9">
+        <v>46247.814390625004</v>
+      </c>
       <c r="D173" s="9">
-        <v>46224.25045253472</v>
+        <v>46247.814415127315</v>
       </c>
       <c r="E173" s="10" t="s">
         <v>196</v>
@@ -11793,9 +11997,11 @@
       <c r="B174" s="5">
         <v>46162.567320891205</v>
       </c>
-      <c r="C174" s="6"/>
+      <c r="C174" s="5">
+        <v>46247.81439159722</v>
+      </c>
       <c r="D174" s="5">
-        <v>46224.25043752315</v>
+        <v>46247.81441560185</v>
       </c>
       <c r="E174" s="6" t="s">
         <v>196</v>
@@ -11844,9 +12050,11 @@
       <c r="B175" s="9">
         <v>46162.567330034726</v>
       </c>
-      <c r="C175" s="10"/>
+      <c r="C175" s="9">
+        <v>46247.81439208333</v>
+      </c>
       <c r="D175" s="9">
-        <v>46224.25043901621</v>
+        <v>46247.814415995366</v>
       </c>
       <c r="E175" s="10" t="s">
         <v>196</v>
@@ -11895,9 +12103,11 @@
       <c r="B176" s="5">
         <v>46162.567337685185</v>
       </c>
-      <c r="C176" s="6"/>
+      <c r="C176" s="5">
+        <v>46247.8143928125</v>
+      </c>
       <c r="D176" s="5">
-        <v>46224.25044046296</v>
+        <v>46247.81441644676</v>
       </c>
       <c r="E176" s="6" t="s">
         <v>196</v>
@@ -11946,9 +12156,11 @@
       <c r="B177" s="9">
         <v>46162.567344166666</v>
       </c>
-      <c r="C177" s="10"/>
+      <c r="C177" s="9">
+        <v>46247.814393692126</v>
+      </c>
       <c r="D177" s="9">
-        <v>46224.2504419676</v>
+        <v>46247.8144168287</v>
       </c>
       <c r="E177" s="10" t="s">
         <v>196</v>
@@ -11997,9 +12209,11 @@
       <c r="B178" s="5">
         <v>46162.56735135417</v>
       </c>
-      <c r="C178" s="6"/>
+      <c r="C178" s="5">
+        <v>46247.814394710644</v>
+      </c>
       <c r="D178" s="5">
-        <v>46224.25044340278</v>
+        <v>46247.81441721065</v>
       </c>
       <c r="E178" s="6" t="s">
         <v>196</v>
@@ -12048,9 +12262,11 @@
       <c r="B179" s="9">
         <v>46162.5673590625</v>
       </c>
-      <c r="C179" s="10"/>
+      <c r="C179" s="9">
+        <v>46247.81439590278</v>
+      </c>
       <c r="D179" s="9">
-        <v>46224.25044509259</v>
+        <v>46247.814417581016</v>
       </c>
       <c r="E179" s="10" t="s">
         <v>196</v>
@@ -12099,9 +12315,11 @@
       <c r="B180" s="5">
         <v>46162.567366284726</v>
       </c>
-      <c r="C180" s="6"/>
+      <c r="C180" s="5">
+        <v>46247.81439731481</v>
+      </c>
       <c r="D180" s="5">
-        <v>46224.25044643518</v>
+        <v>46247.8144181713</v>
       </c>
       <c r="E180" s="6" t="s">
         <v>196</v>
@@ -12203,7 +12421,7 @@
         <v>0</v>
       </c>
       <c r="U181" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="182" spans="1:21" x14ac:dyDescent="0.25">
@@ -12215,7 +12433,7 @@
       </c>
       <c r="C182" s="6"/>
       <c r="D182" s="5">
-        <v>46226.16815751157</v>
+        <v>46247.81168096064</v>
       </c>
       <c r="E182" s="6" t="s">
         <v>190</v>
@@ -12266,7 +12484,7 @@
       </c>
       <c r="C183" s="10"/>
       <c r="D183" s="9">
-        <v>46226.16815899305</v>
+        <v>46247.81304408565</v>
       </c>
       <c r="E183" s="10" t="s">
         <v>190</v>
@@ -12317,7 +12535,7 @@
       </c>
       <c r="C184" s="6"/>
       <c r="D184" s="5">
-        <v>46226.16815614583</v>
+        <v>46247.81446768518</v>
       </c>
       <c r="E184" s="6" t="s">
         <v>190</v>
@@ -12368,7 +12586,7 @@
       </c>
       <c r="C185" s="10"/>
       <c r="D185" s="9">
-        <v>46226.16816035879</v>
+        <v>46247.814529201394</v>
       </c>
       <c r="E185" s="10" t="s">
         <v>190</v>
@@ -12419,7 +12637,7 @@
       </c>
       <c r="C186" s="6"/>
       <c r="D186" s="5">
-        <v>46226.16816185185</v>
+        <v>46247.814529525465</v>
       </c>
       <c r="E186" s="6" t="s">
         <v>196</v>
@@ -12470,7 +12688,7 @@
       </c>
       <c r="C187" s="10"/>
       <c r="D187" s="9">
-        <v>46226.16814340278</v>
+        <v>46247.81420626157</v>
       </c>
       <c r="E187" s="10" t="s">
         <v>196</v>
@@ -12521,7 +12739,7 @@
       </c>
       <c r="C188" s="6"/>
       <c r="D188" s="5">
-        <v>46226.16814550926</v>
+        <v>46247.814529386575</v>
       </c>
       <c r="E188" s="6" t="s">
         <v>196</v>
@@ -12572,7 +12790,7 @@
       </c>
       <c r="C189" s="10"/>
       <c r="D189" s="9">
-        <v>46226.168146909724</v>
+        <v>46247.81452946759</v>
       </c>
       <c r="E189" s="10" t="s">
         <v>196</v>
@@ -12623,7 +12841,7 @@
       </c>
       <c r="C190" s="6"/>
       <c r="D190" s="5">
-        <v>46226.168148275465</v>
+        <v>46247.81420597222</v>
       </c>
       <c r="E190" s="6" t="s">
         <v>196</v>
@@ -12674,7 +12892,7 @@
       </c>
       <c r="C191" s="10"/>
       <c r="D191" s="9">
-        <v>46226.16814969908</v>
+        <v>46247.81420606481</v>
       </c>
       <c r="E191" s="10" t="s">
         <v>196</v>
@@ -12725,7 +12943,7 @@
       </c>
       <c r="C192" s="6"/>
       <c r="D192" s="5">
-        <v>46226.16815109954</v>
+        <v>46247.81420664352</v>
       </c>
       <c r="E192" s="6" t="s">
         <v>196</v>
@@ -12776,7 +12994,7 @@
       </c>
       <c r="C193" s="10"/>
       <c r="D193" s="9">
-        <v>46226.16815254629</v>
+        <v>46247.81452969907</v>
       </c>
       <c r="E193" s="10" t="s">
         <v>196</v>
@@ -12925,7 +13143,7 @@
         <v>0</v>
       </c>
       <c r="U195" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="196" spans="1:21" x14ac:dyDescent="0.25">
@@ -13192,7 +13410,7 @@
       </c>
       <c r="C201" s="10"/>
       <c r="D201" s="9">
-        <v>46227.168836944446</v>
+        <v>46247.81420716435</v>
       </c>
       <c r="E201" s="10" t="s">
         <v>196</v>
@@ -13600,7 +13818,7 @@
         <v>0</v>
       </c>
       <c r="U208" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="209" spans="1:21" x14ac:dyDescent="0.25">
@@ -14275,7 +14493,7 @@
         <v>0</v>
       </c>
       <c r="U221" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="222" spans="1:21" x14ac:dyDescent="0.25">
@@ -14950,7 +15168,7 @@
         <v>0</v>
       </c>
       <c r="U234" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="235" spans="1:21" x14ac:dyDescent="0.25">
@@ -15696,7 +15914,7 @@
         <v>0</v>
       </c>
       <c r="U248" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="249" spans="1:21" x14ac:dyDescent="0.25">
@@ -15759,7 +15977,7 @@
         <v>0</v>
       </c>
       <c r="U249" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>